<commit_message>
fix truncated posts from archive
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4675" uniqueCount="4675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4895" uniqueCount="4895">
   <si>
     <t>日付</t>
   </si>
@@ -30059,6 +30059,2201 @@
 ・料理
 ・旅行
 ・スポーツ</t>
+  </si>
+  <si>
+    <t>「筋トレの時間がない」は甘え。
+俺が一日10時間労働の中、90分の筋トレができる理由はこれ↓
+【やめるべき行動】
+・ポルノ
+・ゲーム
+・女を追う
+・食事に迷う
+・服装に迷う
+・LINEを続ける
+・目的なしSNS
+【マルチタスク】
+・授業or仕事中に副業
+・散歩中、考え事
+・移動中、音声学習</t>
+  </si>
+  <si>
+    <t>「筋トレの時間がない」は甘え。
+俺が一日10時間労働の中、90分の筋トレができる理由はこれ↓
+【やめるべき行動】
+・ポルノ
+・ゲーム
+・女を追う
+・食事に迷う
+・服装に迷う
+・LINEを続ける
+・目的なしSNS
+【マルチタスク】
+・授業or仕事中に副業
+・散歩中、考え事
+・移動中、音声学習</t>
+  </si>
+  <si>
+    <t>自己満男磨き(笑)と呼ばれている習慣を擁護します。
+・オナ禁
+→健康的な射精頻度の方には効果なし。
+でもオナ猿には効果的。
+・ED改善
+・自己管理能力の向上
+・ジヒドロテストステロンの抑制
+個人的には2日以上やるとびんこち〇ち〇になるため、
+セスクの前にやっておきたい。
+【瞑想】</t>
+  </si>
+  <si>
+    <t>自己満男磨き(笑)と呼ばれている習慣を擁護します。
+【オナ禁】
+→健康的な射精頻度の方には効果なし。
+でもオナ猿には効果的。
+・ED改善
+・自己管理能力の向上
+・ジヒドロテストステロンの抑制
+個人的には2日以上やるとびんこち〇ち〇になるため、
+セスクの前にやっておきたい。
+【瞑想】</t>
+  </si>
+  <si>
+    <t>🌟清潔感改善リスト
+以下の方法で完璧にしろ
+・腕毛、指毛、その他体毛→家庭用脱毛
+・唇→血色のよくなるリップ（UNOがおすすめ）
+・脇毛→剃る
+・イチゴ鼻→毎日入浴＆週１サウナ
+・もみあげ→逆三角形を維持
+・髪→5000円以上のメンズカット
+・眉毛→週3回手入れ
+・髭→レーザー脱毛</t>
+  </si>
+  <si>
+    <t>＃今日の積み上げ
+おはようございます☁
+AM
+✅朝散歩
+✅家事（ベッドメイク、食洗器）
+✅目標整理
+✅ポスト3つ作成
+✅英語学習
+PM
+✅英語学習
+✅筋トレ→肩、三頭筋
+✅バルク飯
+カフェイン断ち二日目ですが、睡眠がめちゃ深いです
+このまま1週間継続する予定
+体重は順調に増えてます
+今、62.7kg</t>
+  </si>
+  <si>
+    <t>＃今日の積み上げ
+おはようございます☁
+AM
+✅家事
+✅英語学習　全パート完全攻略
+✅ポスト3つ作成
+PM
+✅英語学習　全パート完全攻略
+✅懸垂
+✅スクワット
+今日からTOEIC本番の10/27まで一日5時間は英語学習に割きます
+カフェインは後1週間くらいデトックス</t>
+  </si>
+  <si>
+    <t>＃今日の積み上げ
+おはようございます
+AM
+✅家事　(食器洗い、洗濯、掃除機)
+✅バルク飯買い出し　
+✅金フレ　200語
+PM
+✅TOEIC 全パート攻略PT.5
+✅️16:00懸垂と脚トレ
+昨日サボってしまった脚トレと懸垂は必ずやる
+弱いって俺　体調を言い訳にしてしまった</t>
+  </si>
+  <si>
+    <t>🌟弱者男性と強者男性の違い
+趣味編
+🔵弱者男性
+・スナック菓子
+・AV鑑賞
+・漫画喫茶
+・カードゲーム
+・鉄道
+・パチンコ
+・スポーツ観戦
+・SNSでレスバ
+・マニアックなゲーム
+🔴強者男性
+・ナッツ
+・美女とSEX
+・カフェ巡り
+・旅行、温泉
+・読書
+・スポーツ
+・筋トレで先週の自分と格闘</t>
+  </si>
+  <si>
+    <t>🌟女に格上認定される方法
+・女＜＜＜＜夢
+・小さな頼みごとをする
+・他の女を匂わせる
+・ハプニングに冷静に対応
+・褒められてもあっさり
+・ブスやチー牛にも優しく接する
+・既読無視
+・ヘラヘラしない
+・即決
+・リーダーシップを取る
+・イケてる友達と絡む
+・当たり前のように奢る</t>
+  </si>
+  <si>
+    <t>🌟男磨き初心者が知っておくべき真実
+・女は上位20％の男以外興味ない
+・ベンチプレス平均は43kg
+・筋トレは初心者の方が成果が出る
+・筋肉質は統計的にモテる
+・金、地位より身体、顔、コミュ力
+・コミュ力はインプットゲー
+・オナ禁は無意味
+・ポルノ断ちは効果絶大
+・整形なしでも顔は変わる</t>
+  </si>
+  <si>
+    <t>強者男性と弱者男性との違い10選
+マインドセット編
+🔴強者男性
+①失敗前提で行動
+②積極的に人に頼る
+③成果は雪だるま式
+④圧倒的エゴイスト
+⑤「まだ出来てないだけ」
+⑥遺伝＜＜＜＜環境＆努力
+⑦40代にピークを持っていく
+⑧経年進化
+⑨ビッグマウス
+⑩目立ってなんぼ
+🔵弱者男性
+①成果を急ぐ</t>
+  </si>
+  <si>
+    <t>スマホ依存症をスマホ依存対策アプリで治そうとしてる内は無理だよ
+バーでアルコール依存症自助会を開催してるようなのも
+重要なのは
+①スマホを物理的に隔離する
+→タイムロック、郵便ポストに入れる
+②自己研鑽に没頭
+筋トレ、資格、女、読書
+③ネットへの執着をなくす</t>
+  </si>
+  <si>
+    <t>【モテの公式】
+モテ＝試行回数×魅力度
+・試行回数とは女へのアプローチの事。
+ナンパ、マチアプ、職場、学校などで女にアプローチする回数。
+・魅力度とは男の魅力
+顔、身体、ステータス、経済力、コミュ力、特技
+頭が弱い人は試行回数を上げることばかり気にし、魅力度という数値を意識しない。</t>
+  </si>
+  <si>
+    <t>※「必要なサプリ」なんてありません。
+Supplement=不足しているものを補うもの
+なので、そもそも栄養を不足させない事が一番です。
+食材から摂りましょう。
+亜鉛、マルチビタミンなど日本食には不足しがちな栄養素を摂るのはありです。
+僕は亜鉛だけ摂ってます。</t>
+  </si>
+  <si>
+    <t>月90時間を作り出す方法
+※「時間がない」が口癖の人へ
+以下の方法で一日3時間、浮かせるだけ
+・ショート動画SNSを消す
+＋60分
+・起床後スマホやめる
+＋30分
+・食洗器を使う
+＋20分
+・栄養計算し毎日同じ食事
+＋20分
+・ドラム式洗濯機を使う　
+＋10分
+・液体カロリーを摂る
+＋10分</t>
+  </si>
+  <si>
+    <t>男磨きが必要な人の特徴
+※もし以下に一つでも当てはまっていたら、女追うのをやめて男磨き期間を作ってみてほしい。
+・10代
+・童貞
+・夢がない
+・チー牛顔
+・スマホ依存症
+・月収10万以下
+・デブorヒョロガリ
+・経験人数10人以下
+・男から舐められる
+・理想の女とS●Xできていない</t>
+  </si>
+  <si>
+    <t>【2024年上半期の自己投資12選】
+結論：過去一、金を使っているが後悔０
+強者になりたければ、N●SAより自己投資にフルベットしろ
+・レーザー脱毛
+12万円
+・デート
+計10万円
+・一人暮らし
+月6万円
+・食洗器
+5万円
+・Sonyヘッドホン
+5万円
+・縮毛矯正
+2万円
+・タップル
+1万2000円
+・ZARAレザーバッグ</t>
+  </si>
+  <si>
+    <t>【童貞は大きく分けて3種類】
+自分がどこに当てはまるかを客観視し、正しい努力をしろ
+・アッパー型童貞
+→基本エネルギッシュ。だが努力の方向性をことごとく間違えている。
+例：派手髪、酒タバコイキリ、大学デビュー、片っ端から告白、ゴマすり
+成功方法→外見磨き。これに尽きる。</t>
+  </si>
+  <si>
+    <t>簡単に月1万円を取り戻す方法
+※「金がない」が口癖の人へ
+以下の工夫で、ストレスなく月1万円が手に入る
+・外食→自炊
+＋3000円
+・サブスク解約
+＋1000円
+・不良品を売る
+＋1000円
+・キャッシュレス決済
+＋1000円
+・ジャンクフード禁止
+＋1000円
+・図書館利用で電気代節約
+＋1000円</t>
+  </si>
+  <si>
+    <t>🌟筋トレで伸び悩む人がやるべきこと20選
+俺は5年くらい、全く身体が変わらなかった経験をしている。
+でも、以下を意識してから3ヶ月、体重2~3kg増量、記録も毎週更新している。
+ートレーニング改善ー
+①記録を取る
+②重量＜＜＜フォーム
+③ボリューム＜＜＜強度
+④余力は残さない</t>
+  </si>
+  <si>
+    <t>🌟格上感を出すテクニック（笑）はフル無視でOK
+女に対する余裕は自然と生まれてくるもの。
+正しい男磨きをしていれば、作らなくても、勝手に生まれてくる。
+例えば
+返信を遅くする
+→仕事が忙しい、他の女からもメッセージが来る。
+だから返信が自然と遅くなる。</t>
+  </si>
+  <si>
+    <t>【大学生とニートへ】
+今、大学生やニートをやっている人はチャンスだと思った方がいい。
+忙殺されることなく、自分のやりたいことにフルに没頭できるから。
+今、俺は大学生だが年の半分くらいは休日だし、授業も大して出席しなくても単位が取れる。
+なんなら授業を受けつつ、仕事ができる。</t>
+  </si>
+  <si>
+    <t>オナ禁はだけで留まってる奴は甘え。
+オナ禁信者は「筋トレ」「ナンパ」「勉強」「仕事」といった、さらに精神力のいる男磨きから逃げて、何かをやった気になっているだけ。
+あくまでオナ禁は、これらの男磨きをサポートする役割</t>
+  </si>
+  <si>
+    <t>🌟清潔感のセルフケアチェックリスト
+女と会う前に確認必須
+※一つでも、ケアを怠っていたら危機感持て
+ースキンケアー
+☑睡眠食事運動の徹底
+☑保湿
+☑紫外線予防
+☑湯船につかり汗を出す
+ー体毛の処理ー
+☑鼻毛
+☑指毛
+☑顔そり
+☑腕毛
+☑うなじ
+ーヘアケアー
+☑ヘアオイルでパサつき抑える</t>
+  </si>
+  <si>
+    <t>🌟上位1％の男の朝ルーティン8ステップ
+①ベッドメイク
+②体重測定
+③ハイドレーション
+→水＋電解質（塩＋レモン）を500ml
+④ブラックコーヒー
+⑤散歩15分
+⑥ToDo作成
+⑦1~2時間のディープワーク
+⑧筋トレ
+寝てる間に、大量の水分を失ってるから、水分補給はマスト。</t>
+  </si>
+  <si>
+    <t>【春休み突入】
+負け組大学生と勝ち組大学生の違い
+🔵負け組大学生
+・昼に起きる
+・アルバイト三昧
+・モラトリアムを味わう
+・他人を批判、応援する
+・コンビニ飯
+・スクリーンタイム6時間越え
+・四六時中、SNSを見る
+🔴勝ち組大学生
+・6~8時に起きる
+・スキル向上orビジネス</t>
+  </si>
+  <si>
+    <t>非モテと魅力的な男の金の使い方の違い
+🔵非モテ　　　　🔴魅力的な男
+・服に1万円　　　　ジムに1万円
+・マック1000円　　  ステーキ
+・推し活　　　　　   自己投資
+・一人で外食　　　   デートで外食
+・ラーメン500円　　 500円で卵20個 
+・EAA3000円　　　　3000円でクレアチン</t>
+  </si>
+  <si>
+    <t>🌟凡人と上位10%の男の筋トレの違い
+🔵凡人
+・重量にこだわる
+・筋肉よりメンタルが先に負ける
+・インターバル1~2分
+・「限界まで追い込む！」（余力5レップ）
+・パーシャルなし
+・トレ前に入念なストレッチ
+・記録を取らない
+🔴上位10%の男
+・筋肉への刺激にこだわる
+・筋肉が先に負ける</t>
+  </si>
+  <si>
+    <t>🌟凡人と上位10%の男の筋トレの違い
+🔵凡人
+・重量だけこだわる
+・筋肉よりメンタルが先に負ける
+・インターバル1~2分
+・「限界まで追い込む！」（余力5レップ）
+・パーシャルなし
+・トレ前に入念なストレッチ
+・記録を取らない
+🔴上位10%の男
+・筋肉への刺激にこだわる
+・筋肉が先に負ける</t>
+  </si>
+  <si>
+    <t>”非モテな自分を正当化する奴は負ける”
+先日、大学のゼミで
+「女なんて金かかるだけだから必要ない」と典型的な非モテの戯言を言っている奴がいた。
+もちろん、そいつには女はいないし、ヒョロガリ低身長で、どう見ても毎晩シコってる顔の男だ。</t>
+  </si>
+  <si>
+    <t>🌟童貞卒業で変わる価値観15選
+①女は格上男には性格が良い
+②何を言うか✖誰が言うか○
+③セックス＝性的快感＜優越感
+④草食系は雑魚
+⑤筋肉はモテないは嘘
+⑥酔わせなくてもヤれる
+⑦0→1よりも1→10は簡単
+⑧ち○こはデカさより硬さ
+⑨プランの練りすぎは悪手
+⑩下心はタイミング</t>
+  </si>
+  <si>
+    <t>🌟高ポテンシャルな男の特徴
+当てはまってる人は、今は非モテだろうが将来成功する可能性大。
+ーマインドー
+・1~2年の長期プラン
+・「まだ出来てないだけ。」
+・結果は雪だるま式
+・他人を批判or応援しない
+・内省を繰り返す
+ー習慣ー
+・筋トレ週5
+・英語
+・PCFを意識した食事
+・8時間睡眠</t>
+  </si>
+  <si>
+    <t>🌟ヒョロガリのお前に必要な高タンパク食材
+ー動物タンパク質ー(100gあたり）
+・ホエイプロテイン　30g
+・マグロの赤身　　　26g
+・鶏むね肉　　　　　25g
+・鶏もも肉　　　　　25g
+・ステーキ　　　　　22g
+・サバ  　　　　　　  20g
+・卵　　　　　　　　12g
+・ギリシャヨーグルト  9g</t>
+  </si>
+  <si>
+    <t>現代の男はデジタル・ドーパミンとの闘い
+一生、Xスクロールして人生終えたくない奴は読め
+スマホに依存する人と使いこなす人の違い
+🔵スマホ依存症
+・スマホでアラーム
+・「このアプリいつか使うかも」
+・「すぐ返信しないと」通知オン
+・ストレス発散→ゲーム
+・隙間時間にショート動画</t>
+  </si>
+  <si>
+    <t>”格上の男”になるために習慣づけるべき行動
+・即断即決
+・リーダーになる
+・女よりも高い美意識
+・男からの尊敬を集める
+・頼みごとをする
+・前髪を上げる
+・ゆったりとした動作
+・声を1トーン落とす
+・身体をデカくする
+・出会い序盤はプッシュ戦略
+・相手が食いついたらプル戦略</t>
+  </si>
+  <si>
+    <t>”あなたのスマホ依存を誘発するトリガー9選”
+トリガーを排除するだけでスマホ依存は緩和する
+1.暇
+2.通知
+3.精神的疲労
+4.ショート動画
+5.視界にスマホ
+6.自動再生機能
+7.散らかったベッド
+8.低テストステロン
+9.ゲームのログインボーナス
+人間は暇になるとコミュニケーションがとりたくなる。</t>
+  </si>
+  <si>
+    <t>⚠️常習化すると一生非モテになる思考
+9選＆対処法
+（20歳自閉症チー牛の俺が本気で考えていたこと）
+①親ガチャ
+②冷笑主義
+③自己卑下
+④運命の女性
+⑤競争から逃げる
+⑥「大企業に勤めて女を見返すやで！」
+⑦「告白すれば振り向いてくれる！」
+⑧努力の過大評価
+⑨0か100か
+① 親ガチャ
+✖️</t>
+  </si>
+  <si>
+    <t>妄想童貞オナ禁くん（20歳）の俺が本気で信じていたスーパーパワー
+・100日目で逆ナンされる
+・7日目で記憶力10倍
+・精子を貯めると筋肉がつきやすい
+・一発抜いたらテストステロン底落ち
+・オナ禁フェロモンが女を呼び寄せる
+・電車で隣に美女が座ったらオナ禁の効果</t>
+  </si>
+  <si>
+    <t>ホームジムはやめたほうがいい。
+俺は2年前に懸垂バー兼パワーラックとダンベル買った。　
+でも今は扱える重量が大きくなって結局ジムに通ってる。
+当時は「ジムよりお得。外に出なくていい！」だったけど、結局、筋トレ極めるとマシンと家には収まらないダンベルが必要になる。</t>
+  </si>
+  <si>
+    <t>Xのスクロールがやめられない原因＆対処法
+＃スマホ依存
+①通知
+②睡眠不足
+③コミュニケーション不足
+④フィードにエロコンテンツ
+⑤不安を煽るニュース
+⑥ドーパミン過多
+⑦やるべき事をサボっている
+⑧スマホアプリ
+対処法↓
+①通知
+→SNSは時間を取って目的を持ってみる
+②睡眠不足</t>
+  </si>
+  <si>
+    <t>筋トレで自分が何やってるのか分かってない人が多すぎる。
+目的をしっかり定め、逆算してやることをハッキリさせよう。
+目的は大きく分けて3種類。
+「モテボディ」「筋肥大」「重量更新」
+【モテボディ】
+体脂肪率8%～13％を目指す。上半身中心に鍛える。</t>
+  </si>
+  <si>
+    <t>「美人は性格悪い」と感じるのは、あなたに性的な魅力がないからです。
+性的魅力のない男からのアプローチは攻撃に等しい。
+なぜなら10か月妊娠期間を経た上にチー牛の子供を産まさせるわけだから。
+勘違いをさせないために冷たい対応するのは当然。</t>
+  </si>
+  <si>
+    <t>意外とコミュ力はインプットゲーなんだよ。
+よく「コミュ力高めたいなら人と話せ！」とアドバイスする奴がいるがこれはおかしい。
+だってチー牛は人と話せないから困っているわけで。
+まずは人と話さずに、知識を入れてメンタルリハーサルをしていく必要がある。</t>
+  </si>
+  <si>
+    <t>「モテたきゃ金銭的リスク取れ」は嘘。
+チー牛が人並に女を抱けるようになるまでは、ほぼリスクはない。
+実際に童貞捨てるまで俺が取ったリスクは
+・美容室代　7000円/月
+・服をそろえる　約7万円
+・マッチングアプリ　1万2000円
+せいぜい、こんなもん。</t>
+  </si>
+  <si>
+    <t>【孤独でもメンタルを安定させる方法】
+男磨きは孤独との戦いになるので実践してほしい。
+①朝散歩
+②1時間の筋トレ
+③ポジティブ3行日記
+④笑顔を作る
+⑤8時間睡眠
+⑥SNSで成果報告
+孤独だとしても、メンタルが安定していれば、むしろ人生はいい方向に進む。</t>
+  </si>
+  <si>
+    <t>やらかしてしまった時のスイッチング行動
+男磨きは長期で継続するもの。
+「いかにメンブレを減らすか」が重要になってくる
+①スマホ断ち
+②悩みを紙に書きだす
+③長期プランを立てる
+④深呼吸
+⑤無心で散歩
+⑥やらかした原因分析
+⑦ふて寝</t>
+  </si>
+  <si>
+    <t>対人関係は"とにかくギブ"。
+恋愛は「いかに相手をドキドキさせるか」から逆算して考える。
+自己完結男磨きは、それを達成するための手段に過ぎない。
+Xを開始して3週間目。
+俺も目先のインプ得るためではなく、本当に良いと思った情報を人生絶望している男たちに届けたい。</t>
+  </si>
+  <si>
+    <t>⚠️魅力度0で「マチアプ」やってもモテません。
+モテ＝「魅力度」×「試行回数」×「戦略」を意識してください。
+魅力度が0だった場合、試行回数を1000万にしてもモテないです。
+アメリカのTinderの調査では、魅力度下位20%の男のマッチ率は0.1~0.5%だとわかっています。</t>
+  </si>
+  <si>
+    <t>【モテの公式】
+これを意識して「あなたが取り組むべき事」を明確にしましょう。
+簡単に3ヶ月で童貞卒業＆セフレ量産できます。
+モテ＝「魅力度」×「試行回数」×「戦略」
+それぞれ詳しく解説↓
+【魅力度】
+まず童貞が取り組むべきは魅力度向上。</t>
+  </si>
+  <si>
+    <t>【モテの公式】
+これを意識して「あなたが取り組むべき事」を明確にしましょう。
+僕がたった一年で、自閉症チー牛の状態から童貞卒業＆セフレ量産をした方法を共有します。
+モテ＝「魅力度」×「試行回数」×「戦略」
+それぞれ詳しく解説↓
+【魅力度】
+まず童貞が取り組むべきは魅力度向上。</t>
+  </si>
+  <si>
+    <t>「環境のせいにするな」を鵜吞みするな。
+あなたが努力したくてもできないのは「意志力」ではなく明らかに「環境」のせい。
+環境のせいにして環境を変える努力をしよう。
+環境を変える上で意識する事は
+・SNSで誰をフォローするか
+・ネガティブ人間を避ける
+・部屋を綺麗にする</t>
+  </si>
+  <si>
+    <t>感情的な男には継続力がない
+上手くいっている時に「よっしゃー！俺は無敵だ！」となる男は、停滞期に絶望感を味わうからだ。
+停滞期、成果が見えない時期にいかに無心で努力を続けるかが重要。
+継続したいなら勝ってカブトの緒を締めろ。
+そして一喜一憂せず成功要因を冷静に分析しろ。</t>
+  </si>
+  <si>
+    <t>感情的な男には継続力がない
+上手くいっている時に「よっしゃー！俺は無敵だ！」となる男は、停滞期に絶望感を味わうからだ。
+停滞期、成果が見えない時期にいかに無心で努力を続けるかが重要。
+継続したいなら勝ってカブトの緒を締めろ。
+そして一喜一憂せず成功要因を冷静に分析しろ。</t>
+  </si>
+  <si>
+    <t>【過大評価されている男磨き】
+・オナ禁
+・ファッション
+・モテテク
+・高価なスキンケア
+・サプリメント
+・コールドシャワー
+【過小評価されている男磨き】
+・睡眠
+・筋トレ
+・ジャーナル
+・コミュ力向上
+・インスタ運用
+・デート＆ナンパ</t>
+  </si>
+  <si>
+    <t>孤独の中でも、努力を続ける方法
+男磨き3年目の俺が教える、仲間を作らず継続する方法
+「男磨き始めたけど仲間がいない...」みたいな人は試してみて
+【環境づくり】
+・ジムに通う
+・カフェで作業
+・目標をデスクに張る
+・SNSで目標と進捗報告
+・男磨き発信者をフォロー</t>
+  </si>
+  <si>
+    <t>よく男磨き界隈で「完璧主義はやめろ」というが、それは「継続できなくなるくらいなら」前提の話。
+つまり、ベストではなくベター。
+本当にデカいこと成し遂げたいならスティーブ・ジョブズの周りをドン引きさせるキ〇ガイのような完璧主義者にならなくてはいけない。</t>
+  </si>
+  <si>
+    <t>大学生とニートの使える時間はバグ。
+俺はどちらも経験してるから言える。
+ニート時代の2年間で本100冊は読んだ。
+大学生の今は平日の昼間にほぼ貸切状態のジムにも行ける。
+こんな最高な期間は人生で滅多にないから、酒飲んでゲームして適当に女遊びするだけだと絶対に30代で後悔すると思う。</t>
+  </si>
+  <si>
+    <t>⚠️男を腐らせる悪習慣17選
+僕のオナ猿童貞時代は全部、当てはまってました。
+①謙遜
+②満員電車
+③座りすぎ
+④運動不足
+⑤母親に頼る
+⑥競争から逃げる
+⑦ドーパミン中毒
+⑧先延ばし癖
+⑨日光不足
+⑩7時間睡眠以下
+⑪ネガティブ思考
+⑫人の悪口を言う
+⑬人の応援をする
+⑭水分不足（最低1日2L）</t>
+  </si>
+  <si>
+    <t>【外見＝内面】
+「恋愛では外見が良くないと内面は見てくれない。だから外見を磨くべき。」という考えができる時点で、内面も素晴らしい。
+なぜなら、外見を磨く＆キープするには
+・適度な有酸素運動
+・最低週2日の筋トレ
+・忙しい中で7~8時間睡眠
+・栄養バランスの取れた食事
+・月1美容室</t>
+  </si>
+  <si>
+    <t>男磨きで最初に初めるべきなのは筋トレではない。
+”他責思考を捨てること”
+すべてはここから始まる。
+「全部自分のせい」と思えた瞬間に自分を変えようとなるからだ。
+もしあなたが
+「親ガチャが....」
+「友達がいなのは周りが冷たいから」
+「モテないのは男を顔で見る女が悪い」</t>
+  </si>
+  <si>
+    <t>”プライドが低い男は一生成長しない”
+悔しい経験をしても、「まぁ俺は雑魚だから」とすぐに開き直るようでは、自分を変えようとは思えない。</t>
+  </si>
+  <si>
+    <t>"人前で堂々と振舞うために意識すべきこと"
+クラスの一言も喋らないチー牛（20歳）が意識して変えていった事
+【テクニック】
+①ボケる
+②間を空ける
+③軽く微笑む
+④70%アイコンタクト
+⑤目を逸らす時は横を見る
+⑥話すスピードは1.3倍速
+⑦強調したい時はゆっくり
+⑧顎を少し斜め上にして自信を演出</t>
+  </si>
+  <si>
+    <t>「ゲームをやめるとストレスになる😠」って言ってる奴はゲーム中毒脳。
+そりゃドーパミン中毒状態でゲームをやめたら禁断症状が来るでしょ笑　自己正当化でしかない。
+1週間くらいやめて、別の事に熱中してみたら「俺、マジで馬鹿なことやってたな」と思うよ。</t>
+  </si>
+  <si>
+    <t>継続のコツは「質にこだわらず、無理なく続ける」こと。
+これを一カ月くらい続けると、逆にやらないのが気持ち悪く感じるようになる。歯磨きと同じ。
+俺は何やっても三日坊主だったけど、筋トレだけは2年以上続けている。
+最初は「強度はどうでもいいからとりあえず毎日やる」で継続した。</t>
+  </si>
+  <si>
+    <t>「マッチョになりすぎるのは嫌」という気持ちは分かる。
+けど、モテボディを目的に筋トレしてるなら、ボディビルダー向けの情報は見ておいた方が良い。
+なぜなら、ボディビルダーは筋肥大を第一に考えているから。</t>
+  </si>
+  <si>
+    <t>失敗した時に秒速で切り替えることが重要。
+ぶっちゃけ、モチベ上げよりも意識すべき。
+オナ禁信者に多いことだが、失敗した時に「今日は堕ちるとこまで堕ちよう」とすぐ悪い方向に開き直る。
+そうじゃなくて、反省した上で「まぁどうでもいいか。また続けよう。」と切り替えれる奴は強い。</t>
+  </si>
+  <si>
+    <t>あなたの努力量はショボい。
+・週3の筋トレ
+・毎日1時間の副業
+・毎日30分コツコツ英語学習
+こんな努力量は誰でもこなしてるから、並みの結果しか得られない。
+あなたは環境を変えて基準値を上げる必要がある。
+そしたら「自分は甘かった」と感じているようになり、努力の基準値が爆上がりするよ。</t>
+  </si>
+  <si>
+    <t>【カフェイン断ち】
+毎日コーヒー飲んでいる人は定期的にカフェイン断ちしよう
+カフェイン解禁した時の効果が数倍になる。
+俺は毎朝1〜2杯濃度高めのブラックコーヒーを飲むけど、昨日は今日のプレゼンのために抜いてきた。</t>
+  </si>
+  <si>
+    <t>筋肉がモテるの本質9選
+①顔デブ防止
+②健康な雄の象徴
+③セクースリピート率UP
+④肩幅が広がり小顔になる
+⑤テストステロン向上
+⑥脂肪が付きにくくなる
+⑦シンプルコーデが似合う
+⑧男らしい顔つきになる
+⑨ハグ要求率UP
+筋トレはマジで万能。</t>
+  </si>
+  <si>
+    <t>夏から筋トレを始める男は馬鹿
+「海でモテたい」「ムキムキな腕を見せたい」と思って5月6月から始める奴は筋トレを甘く見てる。
+SNSのイケてる身体した男は1ヶ月2か月の努力で作り上げたわけじゃない。普通の男が夏に向けて気合いれてやる筋トレを少なくとも2年継続している。</t>
+  </si>
+  <si>
+    <t>女遊びほど筋肉に悪い活動はないな笑
+大体「酒」「夜更かし」「チートミール」三昧だし、筋トレに集中してるなら月数回に抑えるべき。
+もしくは、出来るだけ健康的に女遊びをしよう。
+俺は絶対に酒を飲まないで、口説くことに決めている。</t>
+  </si>
+  <si>
+    <t>習慣化と脱依存症には"物理的距離"がカギ
+人は近くにあるものに注意を奪われるから、それを利用すれば習慣化も脱依存症も可能。
+【脱依存症の例】
+・スマホ断ち→部屋に充電器を置かない
+・ゲーム断ち → コントローラーを毎回片付ける
+・SNSをやめたい → SNSアプリを遠くに設置
+【習慣化の例】</t>
+  </si>
+  <si>
+    <t>【経験人数を追うな】
+経験人数なんて、母数を増やせばいくらでも増やせるんだよ。マチアプでマッチ率3%くらいあれば、1000スワイプで30人マッチ。そのうちの5人はイケる。
+ある程度、モテるようになったら女追うのをやめて男磨きで次のレベルに行こう。</t>
+  </si>
+  <si>
+    <t>モテるために「女の趣味を理解しろ」というが趣味の話で盛り上がりすぎると趣味友止まりなんだよな。実際、俺は韓国アイドル、美容、ネイルとかガチで興味0。けどそれで困った事はない。なぜなら女を喜ばせる趣味があるから。「料理」「筋トレ」「英語」このへんだと思ってる。</t>
+  </si>
+  <si>
+    <t>ゲームは人生を破壊する。</t>
+  </si>
+  <si>
+    <t>「男磨き(笑)してても対女スキルは育たない」という意見はごもっとも。
+だけど、過去の俺含め絵に描いたようなチー牛が「マチアプ」「ナンパ」やっても結果が出るわけがない。
+普通の会話ですら、まともに相手されないのが現実。</t>
+  </si>
+  <si>
+    <t>努力のミニマリストになれ。
+「毎日10時間作業してやる」←これも素晴らしいこと。
+だけど「10時間本当に集中できているか？」そこを見直してほしい。もし、その答えがNOなら「10時間あるから省エネで適当にやろう」と脳が無意識に思っている。</t>
+  </si>
+  <si>
+    <t>”ビビりな性格”こそがチー牛アクションを取ってしまう原因。
+・嫌われないようゴマすり
+・ジムは怖い→家トレだけ
+・美容室は怖い→チー牛カット
+・低リスク思考→チャレンジできない
+・目が合ったら怖い→ストレートネック
+・「キモがられたらどうしよ」ナンパできない</t>
+  </si>
+  <si>
+    <t>最終的に男磨きは科学的データより本人の体感がすべて。
+「オナ禁」も「朝5時起き」もやってて自分が調子いいならやればいいし、体感がないならやめれば良い。
+科学的根拠は新しい事を始める時の大まかな指針にはなり得るが、あなたに最適なアドバイスをしてくれるものではない。</t>
+  </si>
+  <si>
+    <t>努力のミニマリストになれ。
+「毎日10時間作業してやる」←これも素晴らしいこと。
+だけど「10時間本当に集中できているか？」そこを見直してほしい。もし、その答えがNOなら「10時間あるから省エネで適当にやろう」と脳が無意識に思っている。</t>
+  </si>
+  <si>
+    <t>コミュ力は「何を言うか」より「誰が言うか」が圧倒的に大事。
+俺の初彼女は大学のグループワークで「次、一緒に授業受ける？」ってナンパした。けど、これが男磨き始める前のチー牛顔の俺が言ったらクソキモいよ。</t>
+  </si>
+  <si>
+    <t>”ブス・ババア相手でもいいから童貞卒業しろ”
+理由はセックスに対する幻想を壊し「あ、こんなもんか」思うため。
+この幻想があるとセックスへの渇望で頭がいっぱいになる。この状態で男磨きもクソもない。</t>
+  </si>
+  <si>
+    <t>禁欲というよりも没頭。
+よく男磨き界隈では「オナ禁しろ」「スマホ断て」と言うが、これらは"没頭"によって勝手に達成されるのが理想的。
+オナ禁の日数記録することも素晴らしいこと。実際、俺もやっていた。
+けど、何か一つのことに没頭していればオナ禁のことなんて完全に忘れている。</t>
+  </si>
+  <si>
+    <t>スマホ中毒で「スクロールやめられない」っていう人はメタ認知力が足りてない。
+メタ認知力というのは自分を第3者視点で見る能力。</t>
+  </si>
+  <si>
+    <t>「モテたいなら自己投資」と言っても金の使い方は大事
+俺の今までの自己投資を紹介するから屍を越えてゆけ。
+【無駄だった自己投資】
+・ホームジム
+・家庭用脱毛器
+・高額な服
+・目的なし読書
+・マニアックな資格勉強
+・香水
+【効果的な自己投資】
+・ジム
+・レーザー脱毛</t>
+  </si>
+  <si>
+    <t>とにかく脳死で続けてください。
+1年後には95%はリタイアしてるので、続けるだけで上位5％に入れます。
+「筋トレ」「ビジネス」「ナンパ」どの分野も最初はやり方めちゃくちゃでOK。
+完璧を求めて、達成できずに諦めてしまうよりかは100倍マシなので。</t>
+  </si>
+  <si>
+    <t>”男の自信を作るための小さな積み上げ”
+これを365日、習慣的にできている男に自信がない奴はいない。
+・腹式呼吸
+・1日7000歩
+・ヘアセット
+・立って作業
+・目標を確認
+・ベッドメイク
+・鏡の前で笑顔
+・腹から声を出す
+・毎日小さな目標を達成
+・ポジティブな言い聞かせ
+・筋トレで毎週記録を更新</t>
+  </si>
+  <si>
+    <t>恋愛格差が広がる現代でモテるのが簡単な理由
+理由は努力家が優遇されるようになったから。
+大半の男は
+・現状維持で満足
+・努力が中途半端
+だから、努力で突き抜けることが可能。
+ほとんどの男はポルノ中毒。　例え自分磨きをしていてもせいぜい、大学デビューレベル止まり。</t>
+  </si>
+  <si>
+    <t>非モテがやりがちな無駄な男磨き
+・香水
+・オナ禁
+・自重トレ
+・中性寄せ
+・目的なし読書
+・サプリメント
+・メンズメイク
+・コールドシャワー
+・女の「恋愛テク❤」を聴く
+・クソダサ写真でマチアプ
+中性寄せすると、ゴシップ大好きジャニオタ系女がよってきがち。</t>
+  </si>
+  <si>
+    <t>男磨きは筋トレとオナ禁をしておけばいいわけじゃない。
+①外見
+②清潔感
+③経済力
+④コミュ力
+⑤ステータス
+この5つを総合的に鍛えていく必要がある。
+筋トレなんて外見を磨くための手段でしかないんだよ。
+金稼ぎから逃げてはいけない。</t>
+  </si>
+  <si>
+    <t>【男の自信はポイント制】
+毎日の積み上げがゆるぎない自信を構築する。
+・ナンパ
+・ジムでの1レップ
+・毎日ToDoをこなす
+・自力で金を稼ぐ経験
+・100人の前でプレゼン
+小さな事でも365日間毎日積み上げる事が重要。
+自信がみなぎる魔法の言葉など存在しない
+「根拠のない自信」はハリボテ。</t>
+  </si>
+  <si>
+    <t>【俺の過去（18~20歳）のステータス】
+以下のような底辺でも男磨きで下剋上が可能
+・童貞
+・一重
+・高校中退
+・166cm 55kg
+・2年間ニート
+・バイト経験なし
+・口ゴボチー牛顔
+・偏差値40の高校
+・鬼高いプライドの持ち主
+・陰キャからもいじめられる
+・クラスに一人いた一言も喋らないチー牛</t>
+  </si>
+  <si>
+    <t>【俺の過去（18~20歳）のステータス】
+以下のような底辺でも男磨きで下剋上が可能
+・童貞
+・一重
+・オナ猿
+・高校中退
+・ゲーム中毒
+・ポルノ中毒
+・166cm 55kg
+・2年間ニート
+・バイト経験なし
+・口ゴボチー牛顔
+・偏差値40の高校
+・鬼高いプライドの持ち主
+・陰キャからもいじめられる</t>
+  </si>
+  <si>
+    <t>”鬼高いプライドを捨てるな”
+俺はまさに他人見下し系チー牛だったから
+「陽キャは流行ばっか追って頭悪すぎ」
+「オタク、キモすぎだろ」
+と「俺は他人とは違う」マインドを持っていた。</t>
+  </si>
+  <si>
+    <t>”鬼高いプライドを捨てるな”
+俺はまさに他人見下し系チー牛だったから
+「量産陽キャマッシュだっせぇ」
+「オタク、キモすぎだろ」
+と「俺は他人とは違う」マインドを持っていた。</t>
+  </si>
+  <si>
+    <t>【犠牲なくして成功なし】
+「あれもやりたい、これもやらなきゃ」――そんな欲張りな考えでは、器用貧乏になり、平凡な人生を歩むだけ。
+成功の鍵は “一点集中”。
+人は「時間」「金」「精神」――この3つのリソースを 一つの目標に全振り したとき、最大の力を発揮できる。</t>
+  </si>
+  <si>
+    <t>筋トレの停滞、その原因は「トレーニング」「食事」「睡眠」のどれかにある。
+当てはまる部分を見直し、改善しよう。
+トレーニング編
+☑ 記録を取らない
+☑ 限界（挙上速度が落ちるまで）追い込まない
+☑ フォームを軽視
+☑ 呼吸の質が悪い
+☑</t>
+  </si>
+  <si>
+    <t>男磨きの本質は「魅力度向上」。
+それ以上でも、それ以下でもない。
+男磨きで魅力度上げても、女にアプローチする回数増やさないと意味ないよ。
+だから、いくら男磨きして細マッチョのイケメンになったとしても家に引きこもってるだけじゃモテない。</t>
+  </si>
+  <si>
+    <t>【ノートは第二の脳】
+瞑想は不安を悪化させる。
+思考は静まるどころか、反復的にストレスホルモンを分泌し、不安を増幅させることがある。
+不安を鎮める最も効果的な方法は、ノートに殴り書きすること。
+✔ 1日10分、何でもいいから書け。
+✔ 思考を言語化しろ。頭の中で考えても答えは出ない。
+✔</t>
+  </si>
+  <si>
+    <t>【モテは第一印象がすべて】
+ぶっちゃけ、初対面で女に「真面目だね」と思われたら終わりなんだよな。
+「真面目な人」といつ印象があるとチャラいムーブが取れなくなってしまう。
+結果、女に打診が出来ず恋愛対象として見られなくなる。
+対策方法は
+・最初にボケる
+・外見にチャラい要素を入れる</t>
+  </si>
+  <si>
+    <t>【モテは第一印象がすべて】
+ぶっちゃけ、初対面で女に「真面目だね」と思われたら終わりなんだよな。
+真面目な人認定されるとチャラいムーブが取れなくなってしまう。
+結果、女に打診が出来ず恋愛対象として見られなくなる。
+対策方法は
+・最初にボケる
+・外見にチャラい要素を入れる</t>
+  </si>
+  <si>
+    <t>月90時間を作り出す方法
+※「時間がない」が口癖の人へ
+以下の方法で一日3時間、浮かせるだけ
+・ショート動画SNSを消す
+＋60分
+・起床後スマホやめる
+＋30分
+・食洗器を使う
+＋20分
+・栄養計算し毎日同じ食事
+＋20分
+・ドラム式洗濯機を使う　
+＋10分
+・液体カロリーを摂る
+＋10分</t>
+  </si>
+  <si>
+    <t>「勉強する時間がない」は甘え。
+俺が1日10時間労働しながら、毎日2時間の勉強でTOEIC300点を700点に上げることができた理由はこれ↓
+【やめるべき行動】
+・ダラダラスマホ
+・意味のない飲み会
+・勉強ノウハウだけ調べる
+・目的のない読書
+・完璧主義
+【マルチタスク】
+移動中 →</t>
+  </si>
+  <si>
+    <t>髭が濃い人が脱毛するのはマジでもったいない。
+俺は医療脱毛してるけど、理由は中途半端に薄くて伸ばしてもカッコがつかないから。
+俺も髭が濃かったら山田孝之みたいなイケオジ目指したかったよ。
+髭が濃い人は伸ばして整えろ。
+髭が嫌いな女は相手にしなくていい。</t>
+  </si>
+  <si>
+    <t>【筋トレしていてもヒョロガリ】
+①小食
+②睡眠不足
+③タンパク質少なめ
+④ライバルなし
+⑤気が向いたら筋トレ
+⑥追い込む前に終了
+【筋トレで成果を出す人】
+①3食多めに食べる
+②7、８時間睡眠
+③体重×2gのタンパク質
+④ライバルのいる環境
+⑤週６筋トレ
+⑥極限まで追い込む</t>
+  </si>
+  <si>
+    <t>【スマホはドラッグ】
+スティーブジョブズ本人がiPhoneを持ってなかったことと子供に与えなかったのが何よりの証拠。
+あれほど、ドーパミンを簡単に得られるアイテムは他にない。
+当たり前だけど、スマホ中毒者は「モテ」「仕事」「筋トレ」すべてにおいて中途半端な結果しか出ない。</t>
+  </si>
+  <si>
+    <t>「デブは普通に生きていたらならない」と言うが、むしろ普通に生きているからこそデブになる。
+人類がサバンナで暮らしていた時代、食料は常に不足し、飢餓との戦いだった。
+そんな環境で生き延びたのは「目の前にカロリーがあるならすぐに摂取する」個体だった。</t>
+  </si>
+  <si>
+    <t>テストステロンをMAXにする休日ルーティン
+毎休日こなせば、あなたの活力は3倍になります。
+朝
+6:30　日の出で起床
+→電解質＋水500ml
+7:00　散歩＋コーヒー
+8:00　ディープワーク
+11:00　ジムで筋トレ
+昼
+13:00　卵5個＋亜鉛サプリ
+→食後の散歩
+14:30　仕事
+夜
+19:00</t>
+  </si>
+  <si>
+    <t>「シコるとテストステロン下がる」というが、テス値上げる方法なんてオナ禁以外にいくらでもある。
+「睡眠」「高タンパク食」「筋トレ」「日光」
+これらをないがしろにして「オナ禁万歳！」してる人は本当に良くない。</t>
+  </si>
+  <si>
+    <t>【スピってるけど効果的な自己啓発習慣】
+・笑顔を作る
+・5分間の瞑想
+・寝る前の焚火の音
+・アファメーション
+・ポジティブ3行日記
+・作業中にGamma40Hzを聴く
+この中でも「ポジティブ３行日記」は根暗人間な俺にめっちゃ効果的だった。</t>
+  </si>
+  <si>
+    <t>筋トレ歴7年の俺が教えるサプリメント優先順位
+S
+「ホエイプロテイン」「クレアチン」
+A
+「亜鉛」「マグネシウム」「L-シトルリン」
+B
+「クラスターデキストリン」「Alpha GPC」「β-アラニン」　　　　　　　　　　　　　　　　　　　　 
+C
+「フィッシュオイル」「マルチビタミン」
+D</t>
+  </si>
+  <si>
+    <t>【今すぐやめろ】女がマジで興味のない話題
+※アッパー型コミュ障がやりがち
+・車
+・投資
+・筋トレ
+・バイク
+・ビジネス
+・スポーツ系
+・マニアックなゲーム
+特に「筋トレ」「ビジネス」で頑張っているアピールをしたいのはわかる。</t>
+  </si>
+  <si>
+    <t>自称清潔感がある男VS本当に清潔感がある男
+【自称清潔感のある男】
+・「毎日3回歯磨きします」
+・「服は必ず洗います」
+・「月1で髪切ります」
+・「シャンプーは一日2回」
+・「毎日、お風呂入ってます」
+【本当に清潔感のある男】
+・歯列矯正＆ホワイトニング
+・シンプルコーデ
+・毎日ヘアセット</t>
+  </si>
+  <si>
+    <t>【たった3万円で垢抜けする方法】
+俺が貧乏実家暮らし時代にやったことはこれ↓
+【有料】
+・美容室　　　　　           5,000円/月
+・眉サロン　　　　           4,000円/3ヶ月
+・プロテイン　　　           3,000円/月
+・毎日たまご4個　             3,000円/月
+・ZARAを愛用</t>
+  </si>
+  <si>
+    <t>【孤独でもメンタルを安定させる方法】
+男磨きは孤独との戦いになるので実践してほしい。
+①朝散歩
+②1時間の筋トレ
+③ポジティブ3行日記
+④笑顔を作る
+⑤8時間睡眠
+⑥SNSで成果報告
+孤独だとしても、メンタルが安定していれば、むしろ人生はいい方向に進む。</t>
+  </si>
+  <si>
+    <t>1年間、身体が変わらなかった俺が家でやっていたクソトレ
+結論：腕立て30回できるなら早くジム行け。
+・記録しない
+・腕立て伏せ50回
+・浅いスクワット
+・リュックにペットボトル入れてスクワット
+・床でベンチプレス
+・反動を使いまくる
+・パワーグリップなしデッドリフト</t>
+  </si>
+  <si>
+    <t>【20代で習慣化しておきたい男磨き】
+これを30代からやろうとしても、重い腰が上がらない。
+・副業
+・英語
+・ジム
+・ナンパ
+・SNS発信
+・毎月1冊読書
+・朝のディープワーク
+・外見投資
+・海外旅行
+特に「ジム」「SNS発信」「海外旅行」は勢いでしかできない。</t>
+  </si>
+  <si>
+    <t>【モテたければ、2~3年モテを捨てろ】
+目先のモテのために使ってる金はすべて「ジム」「ビジネス」に回せ。
+ヒョロガリ低収入の状態で「マッチングアプリ」「ブランド品」「パーティ」「5,000円の美容室」「香水」これらは全部無駄。
+本質的なレベル上げに使うべき。</t>
+  </si>
+  <si>
+    <t>減量期はタンパク質を多めに摂りましょう。
+僕の場合だと、身長×1.2gで約200g
+理由は身体がタンパク質で不足してるエネルギーを補うからです。
+減量中は炭水化物を減らすと思います。</t>
+  </si>
+  <si>
+    <t>【最速でモテを手にする10ステップ】
+※僕が今からチー牛時代に戻ったらこうします。
+①マチアプで惨敗する→現実を知る
+②Xで男磨きアカ開設
+③依存症克服（ゲーム、ポルノ、SNS）
+④清潔感を100点にする
+⑤筋トレ習慣化（自重でもOK）
+⑥フェイストレーニング
+⑦シンプルコーデ</t>
+  </si>
+  <si>
+    <t>【過大評価されている男磨き】
+・オナ禁
+・ファッション
+・モテテク
+・高価なスキンケア
+・サプリメント
+・コールドシャワー
+【過小評価されている男磨き】
+・睡眠
+・筋トレ
+・ジャーナル
+・コミュ力向上
+・インスタ運用
+・デート＆ナンパ</t>
+  </si>
+  <si>
+    <t>意外とコミュ力はインプットゲーなんだよ。
+よく「コミュ力高めたいなら人と話せ！」とアドバイスする奴がいるがこれはおかしい。
+だってチー牛は人と話せないから困っているわけで。
+まずは人と話さずに、知識を入れてメンタルリハーサルをしていく必要がある。</t>
+  </si>
+  <si>
+    <t>【若い女にモテたいなら「本能」に刺させ】
+小学生の女の子って「年収いくら？」のノリで「50m走何秒？」とか聞いてくるよね？
+実はこれ、バカにできない。
+なぜなら、本能的に正しいから。
+若い女は理屈じゃなく「本能で感じる強い男」に惹かれる。</t>
+  </si>
+  <si>
+    <t>「明日でいいや」を繰り返す人は1年後も同じ事で悩む。
+今年こそ「筋肉をつける」「童貞卒業する」「副業で稼ぐ」と全く同じことを来年の今の時期に悩む事になる。
+「重い腰が上がらない」とか言ってる場合じゃない。</t>
+  </si>
+  <si>
+    <t>【ポルノ断ちとか言ってる奴は二流】
+こんな発信してるけど、俺も3ヶ月前にゲーム依存発症してたし、今でもポルノを見る。
+そんな俺が言える事。
+それは「依存している状態」ではなく「依存してやるべきことが手につかない状態」こそが問題。</t>
+  </si>
+  <si>
+    <t>【休日モーニングルーティン】
+オンラインで稼ぐために私がやっていること
+本気で結果を出したい人は見て
+6:00起床
+・ベッドメイク
+・30分散歩
+・水分補給（塩＋レモン＋水500ml）
+・シャワー
+7:00
+・ブラックコーヒー
+・朝食プロテイン
+・ディープワーク10:30まで
+9:30</t>
+  </si>
+  <si>
+    <t>あなたの努力量はショボい。
+・週3の筋トレ
+・毎日1時間の副業
+・毎日30分コツコツ英語学習
+こんな努力量は誰でもこなしてるから、並みの結果しか得られない。
+あなたは環境を変えて基準値を上げる必要がある。</t>
+  </si>
+  <si>
+    <t>【ルーティンを死守しろ】
+俺の3か月間の発信活動で学んだ事を共有します。
+【ルーティン無視生活】
+・昼12時起きでスマホ2時間
+・仕事時間たった2時間
+・睡眠不足
+・ジムでクソトレ
+・やることに迷う
+・ショート動画中毒
+【ルーティン死守生活】
+・朝7時から仕事
+・仕事時間8~10時間
+・8時間睡眠</t>
+  </si>
+  <si>
+    <t>ルーティンを死守する方法
+怠惰な俺がルーティンを守れるようになった方法
+・就寝・起床時間を固定
+・予定を詰めすぎない
+・SNSは主に発信のみ
+・目的を持ちSNSを見る
+・朝コーヒー
+・朝散歩3,000歩
+・朝2時間のディープワーク
+・夜に明日のToDoを書く
+・ゲームはしない
+・作業はカフェor図書館</t>
+  </si>
+  <si>
+    <t>ゲーム中毒を克服するためにやったこと
+※俺はゲーム中毒で高校中退してる
+・瞑想
+・読書に熱中
+・スマホなし散歩
+・アカウントごと消す
+・期間を決めて禁止
+・郵便ポストにコントローラー
+・現実世界でレベル上げ
+・ご褒美でゲームをやる</t>
+  </si>
+  <si>
+    <t>【孤独でもメンタルを安定させる方法】
+男磨きは孤独との戦いになるので実践してほしい。
+①日光
+②笑顔
+③SNS断ち
+④8時間睡眠
+⑤自己中になる
+⑥高強度の筋トレ
+⑦ポジティブ3行日記
+孤独だとしても、メンタルが安定していれば、むしろ人生はいい方向に進む。</t>
+  </si>
+  <si>
+    <t>【筋トレ前の食事9選】
+※全部コンビニで買えます
+①バナナ
+②肉まん
+③三食団子
+④全粒粉パン
+⑤ドライフルーツ
+⑥白米
+⑦オートミール
+⑧フルーツスムージー
+⑨ギリシャヨーグルト
+これらは筋トレ前1～2時間前に食べてください</t>
+  </si>
+  <si>
+    <t>「モテるため」で止まっている奴は浅い。
+結局、人生の目的は「自分が幸せになる」こと。
+モテは他人軸で主体性がない。
+モテるために「女の趣味を学ぶ」「女ウケのいい趣味を作る」「過度な外見投資」
+これをやってて本当に楽しいか？って話。
+もちろん、幸せになるには「モテ」は重要な要素。</t>
+  </si>
+  <si>
+    <t>「女を忘れて男磨き」は飽きるほどS〇Xしないと無理
+なぜなら、童貞は「S〇X出来たら最高なんだろうな」という幻想を抱いているから。
+常にS〇Xに頭が支配されている状態。
+自分も3年前はそうだった。
+でも、飽きるほどSEXすることで、この幻想が壊せた。
+そして、7か月前に女を切ってから</t>
+  </si>
+  <si>
+    <t>【筋トレ界の矛盾】
+筋トレ発信者で、「科学的根拠が…」とか言う人は多いが、実は何も考えずに地方大会でガチで頑張ってる野球部の方がデカい。
+もちろん、科学的根拠は大切。でも、それ以上に大事なのは
+・食事量
+・筋トレ量
+・睡眠時間
+この３つをしっかりこなすこと。</t>
+  </si>
+  <si>
+    <t>男磨きの本質は「魅力度向上」。
+それ以上でも、それ以下でもない。
+男磨きで魅力度上げても、女にアプローチする回数増やさないと意味ないよ。
+だから、いくら男磨きして細マッチョのイケメンになったとしても家に引きこもってるだけじゃモテない。</t>
+  </si>
+  <si>
+    <t>【筋トレ】神サプリとゴミサプリ
+ゴミサプリに月4,000円払うなら、ジムの民度に金を払え
+【神サプリ】
+・プロテイン
+・クレアチン
+・プレワークアウト
+・クラスターデキストリン
+・マグネシウム
+・整腸剤
+【ゴミサプリ】
+・EAA
+・BCAA
+・HMB（き〇しん）
+・ダイエットサプリ（成分不明なもの）</t>
+  </si>
+  <si>
+    <t>【ジムの民度に金を払え】
+最近、「月額たったの3,000円！」みたいな激安ジムが増えてるけど、本気でカッコイイ身体を作りたいなら、やめておけ。
+理由は
+・混雑でまともに筋トレできない
+・スマホ中毒者がマシンを占領
+→注意するスタッフはいない
+・ガチ勢は引かれる
+・シャワーがない</t>
+  </si>
+  <si>
+    <t>サボった翌日に「昨日の分も取り返そう」とか考えるの、やめた方がいい。
+「昨日サボったから、今日は2日分やろう！」
+──この思考が一番まずい。ハードルが上がって、またサボる未来が見える。
+怠惰な人間が、いきなり倍の努力なんてできるわけない。
+だからこそ大事なのは、</t>
+  </si>
+  <si>
+    <t>「静寂」を使えば、スマホ依存症を治せる。
+理由は、理性を支配する「前頭葉」が発達するから。
+具体的に「静寂」とは
+・10分瞑想
+・無音で作業
+・目を閉じて歯磨き
+・スマホなしで散歩
+・読書に没頭
+・朝はスマホを触らない
+一言で言えば「ながら〇〇」をやめること。</t>
+  </si>
+  <si>
+    <t>あなたが不幸なのは「デジタル依存症」のせいです。
+・劣等感→SNS依存
+・集中できない→ショート動画依存
+・女と話せない→ポルノ依存
+・努力できない→ドーパミン依存
+・不眠→スマホ依存
+・思考できない→生成AI依存
+・時間がない→ゲーム依存</t>
+  </si>
+  <si>
+    <t>すべて環境のせいにしろ。
+そして、環境に死ぬほどこだわれ。
+・SNSで誰を見るか
+・食べるもの
+・寝る場所と時間
+・話す人間
+・作業デスク
+・部屋の音・光・温度
+・ジム選び
+「努力ができない」のは、意思が弱いからじゃない。
+「ビジョンに合わない環境」にいるからだ。</t>
+  </si>
+  <si>
+    <t>【努力中毒の環境づくり】
+人は距離が近いものに依存する。
+これを逆手に取ると
+・本をデスクに置く
+・目標をスマホの壁紙に
+・目標をデスクに張る
+・見える場所にサプリ
+・歩いていけるジム
+これらは、理にかなっている。
+人は近くにあるけど、着手してないと罪悪感を感じるもの。</t>
+  </si>
+  <si>
+    <t>チー牛は何も考えずに、身体だけ鍛えろ。
+余裕で、7割の悩みは解決する。
+・男に舐められる→ヒョロガリだから
+・女にモテない→ヒョロガリだから
+・自信がない→ヒョロガリだから
+・服が似合わない→ヒョロガリだから
+・コミュ障→ヒョロガリだから
+・鬱っぽい→筋トレしないから</t>
+  </si>
+  <si>
+    <t>初心者が筋トレを"習慣化"するコツ3選
+①1%の成長
+②モテるためにやる
+③自宅トレから始める
+④身体を写真に残す
+⑤トレーニングノートを書く
+最初は「モテるため」でOk。
+俺も最初は、モテるために自宅のトレーニングマットで腕立て伏せすることから始めた。
+そして、成長を実感することが大事。</t>
+  </si>
+  <si>
+    <t>初心者が筋トレを"習慣化"するコツ5選
+①1%の成長
+②モテるためにやる
+③自宅トレから始める
+④身体を写真に残す
+⑤トレーニングノートを書く
+最初は「モテるため」でOk。
+俺も最初は、モテるために自宅のトレーニングマットで腕立て伏せすることから始めた。
+そして、成長を実感することが大事。</t>
+  </si>
+  <si>
+    <t>【ガチアスペの会話の特徴】
+全部、チー牛時代の私がやっていた会話です。
+キモいのでやめましょう。
+✅事実だけを重視する
+「科学的には」などを多用。
+感情的やりとりよりも、情報の正確性を優先。
+✅言葉の選び方が独特
+伝わらない言い回しを使う。
+細かなニュアンスを形容できる表現を選ぶ。</t>
+  </si>
+  <si>
+    <t>【マインドフルネスの方法】
+スクロール病の人は試して
+・歯磨き中「歯を磨くこと」だけを考える
+・散歩中「足の裏の感覚」だけに集中する
+・食事中は「味」「匂い」「温度」に意識を向ける
+・風呂にスマホを持ち込まない
+・スマホを見る前に「深呼吸3回」してから開く</t>
+  </si>
+  <si>
+    <t>モテるために筋トレをする男が成長しない理由↓
+🏳️‍🌈🤓「追い込むと歯を食いしばってエラが張る！」
+🏳️‍🌈🤓「脂質と塩分はむくみの原因だ！」
+🏳️‍🌈🤓「体脂肪率は10%をキープ！」
+🏳️‍🌈🤓「細い方が服が似合んだよね。」
+🏳️‍🌈🤓「米は糖質。美容の敵だ！」</t>
+  </si>
+  <si>
+    <t>「明日でいいや」を繰り返す人は1年後も同じ事で悩む。
+今年こそ「筋肉をつける」「童貞卒業する」「副業で稼ぐ」と全く同じことを、来年の今の時期に悩む事になる。
+「重い腰が上がらない」とか言ってる場合じゃない。</t>
+  </si>
+  <si>
+    <t>人を見下す性格は、実は野心の強さの表れ。
+「絶対にこうはなりたくない」という強烈な反発心が、見下しの感情を生む。成功者の多くは、誰かを見下す気持ちを持っている。
+それは単なる性格の悪さではなく、負けたくないという強いエネルギーだ。</t>
+  </si>
+  <si>
+    <t>【アスペがコミュ障を治す5ステップ】
+※すべて私の実体験です。
+①見た目を変える
+人は“他人の期待”に沿って振る舞う（ピグマリオン効果）。
+チー牛みたいな見た目をしてると、周囲に「陰キャ」と思われ、それに合わせた行動をとってしまう。
+まずは見た目を整える。そこがスタートライン。</t>
+  </si>
+  <si>
+    <t>「筋トレよりも食べるのが苦手」なら活動量を見直せ
+1日中歩きまくって、1レップも挙がらなくなるまで高強度の筋トレをしていたら、否が応でも食べたくなる。
+理論的には、食べるから高強度の筋トレできるが正しい
+でも、俺含めてヒョロガリ体質な人は、運動は好きだけど、食べることがマジで嫌い。</t>
+  </si>
+  <si>
+    <t>「オナ禁に執着している男」は、たった一回の射精でテストステロンが下がってしまうクソ雑魚。
+・8時間睡眠
+・週5筋トレ
+・PCFを意識した食事
+・勝利する経験
+・仕事に没頭する
+毎日こなせば、シコりまくってようが関係ない。
+オナ禁神経症になるな。
+英雄は色を好む。</t>
+  </si>
+  <si>
+    <t>【湯シャンの真実】
+私が1年試行錯誤して分かったこと
+❌デメリット
+・臭い
+・整髪料は落ちない
+・最初の方、かゆすぎ
+✅メリット
+・髪質は良くなる
+・湿気に強い髪になる
+・皮脂の分泌量は段々減る
+・かゆみは2週間でなくなる
+・ヘアオイルはいらなくなった</t>
+  </si>
+  <si>
+    <t>【個人的にムダだった自己投資・男磨き】
+同じミスをしてほしくない。屍を越えてゆけ。
+①髭脱毛
+→伸ばして長さを整えろ
+②オナ禁
+→効果があるのはオナ猿のみ
+③なんちゃってホームジム
+→金の無駄。ジムに行け
+④モーニングルーティン
+→散歩して水飲んだら、さっさと作業しろ</t>
+  </si>
+  <si>
+    <t>【アスペがやりがちな恋愛上のミス】
+俺がアスペを自覚する前に犯していたミス
+・自分語り＝コミュ力
+・会話＝議論
+・無表情
+・話し方＜＜＜話す内容
+・外見＜＜＜性格
+・共感＜＜＜真実
+・相手への興味0
+・IQ＝150/EQ＝0
+対処法は、まず自分を理解する事。
+自分を理解すれば、</t>
+  </si>
+  <si>
+    <t>月90時間を作り出す方法
+※「時間がない」が口癖の人へ
+以下の方法で一日3時間、浮かせるだけ
+・ショート動画SNSを消す
+＋60分
+・起床後スマホやめる
+＋30分
+・食洗器を使う
+＋20分
+・栄養計算し毎日同じ食事
+＋20分
+・ドラム式洗濯機を使う　
+＋10分
+・液体カロリーを摂る
+＋10分</t>
+  </si>
+  <si>
+    <t>優しい男性はモテます。
+でも、優しさを”ギャップ”として使えない男性はモテません。
+極端な話
+「ブレイキングダウンに出てくるような男」
+「その辺にいる草食系大学生」
+両者が同じ優しいさを女性に提供しても、評価はガラッと変わります。</t>
+  </si>
+  <si>
+    <t>【弱者男性化してしまう23の習慣】
+◆生き方
+・受動型
+・他責思考
+・🤓「金稼いで女を見返すやで！」
+・長期的快楽＜＜＜短期的快楽
+・男磨き陰キャ
+・行動＜＜＜準備
+・他人を応援（推し活、スポーツ観戦）
+・自己主張しない
+◆見た目
+・口呼吸
+・巻き肩
+・ヒョロガリ
+・ストレートネック</t>
+  </si>
+  <si>
+    <t>バルクアップしたいなら“カロリー計算”は必須。
+この4ステップだけ覚えとこう↓
+① TDEEを出す（TDEEでググれば即）
+→ “1日どれだけ食えば体重が増減しないか”がわかる。
+② 目標摂取カロリーを決める
+→ 増量ならTDEE＋300～500kcal。まずはこれでOK
+③ MyFitnessPalに食事を記録
+→</t>
+  </si>
+  <si>
+    <t>自称清潔感がある男VS本当に清潔感がある男
+【自称清潔感がある男】
+・「毎日3回歯磨きします」
+・「服は必ず洗います」
+・「月1で髪切ります」
+・「シャンプーは一日2回」
+・「毎日、お風呂入ってます」
+【本当に清潔感がある男】
+・歯列矯正＆ホワイトニング
+・シンプルコーデ
+・毎日ヘアセット</t>
+  </si>
+  <si>
+    <t>【目的を手段化しろ】
+確かに「手段を目的化するな」は一理ある。
+間違った方向で自己満に走ったら、ただの遠回り。
+でも一方で、目的のための“やっつけ作業”でやってる限り、限界が来る。
+例えば、
+・「モテるための筋トレ」をしてる男が、
+ 筋トレに恋してるボディビルダーには勝てない。</t>
+  </si>
+  <si>
+    <t>【手段を目的化しろ】
+確かに「手段を目的化するな」は一理ある。
+間違った方向で自己満に走ったら、ただの遠回り。
+でも一方で、目的のための“やっつけ作業”でやってる限り、限界が来る。
+例えば、
+・「モテるための筋トレ」をしてる男が、
+ 筋トレに恋してるボディビルダーには勝てない。</t>
+  </si>
+  <si>
+    <t>デジタルミニマリストのルール10カ条
+「デジタル依存をやめて努力に没頭したい」と言う人だけ見て👇
+①通知は全部オフ
+→メッセージはまとめて返す
+②1日3時間、“完全オフライン”を確保せよ
+→「無」が脳のクリエイティビティを覚醒させる
+③朝のスマホは"毒入りのコーヒー"</t>
+  </si>
+  <si>
+    <t>【あなたが時間貧乏な理由10選】
+※「時間がない」が口癖の人は見て
+① マルチタスク信者
+→脳の切り替えコストが積み重なって、一日が溶ける
+② 完璧主義で着手できない
+→やる前に整えすぎて、結局手が動かない。
+③ AIを頑なに使わない
+→単純作業はすべてAIに投げればいい。
+④</t>
+  </si>
+  <si>
+    <t>男磨きで絶対に気をつけるべきは、
+「誰でも」「簡単に」「自宅で5分！」
+みたいな“甘い言葉”に釣られないこと。
+特に筋トレ系の情報
+その甘い言葉は「お前を強くするため」ではなく
+「サプリを買わせるため」に投げられていることが多い。
+甘い言葉＝慰め、セールス
+厳しい言葉＝真実</t>
+  </si>
+  <si>
+    <t>お前が女性経験ゼロなら、やるべきことはシンプル。
+① 圧倒的な節制
+② 浮いた金と時間を、すべて“男磨き”にぶち込む
+たったこれだけのループでいい。
+「自己投資」って聞くと、大金を積むイメージかもしれない。</t>
+  </si>
+  <si>
+    <t>男磨きしてる真面目な人は肩の力を抜こう。
+俺も普通にシコるし筋トレもサボる。
+「先週と比べて退化したな」なんてことはザラにある。
+でも1カ月、半年単位で成長していればOKという考えを持ってるから「落ちることまで落ちよう」とはならない。</t>
+  </si>
+  <si>
+    <t>最近「オナ禁なんて意味ない。モテには直結しない」という論調が増えているが、
+ 明らかにオナ禁が必要な弱者男性は存在する。
+オナ禁は確かに「0 → ＋」にはならない。
+だが、「マイナス → 0」には確実にしてくれる。
+クーラーの効いたイカ臭い部屋で、終日シコってるオナ猿は、まずはオナ禁。</t>
+  </si>
+  <si>
+    <t>モテる男は「女なんてどうでもいい」と言い、  
+高学歴は「学歴なんて関係ない」と言い、  
+金持ちは「金で幸せは買えない」と言う。  
+執着を捨てるには、  
+一度、飽きるほど手にするしかない。  
+非モテは「俺は女なんていらない。自己実現だ！」と口では言う。</t>
+  </si>
+  <si>
+    <t>「ジムに行く金がない」と言う男には腹が立つ。
+大体「自販機」「洋服代」「8000円の美容室」で浪費しているわけで、金がないというよりも、筋トレの優先度が低いだけ。
+俺みたいな貧乏大学生は
+・水は水道水
+・カロリー計算して自炊
+・シャワーはジムで
+・1000円カットorセルフ
+・電気つけない</t>
+  </si>
+  <si>
+    <t>男磨きは「魅力を最大化して女とヤリまくる」なんていう陳腐なコンセプトじゃない。  
+チー牛が“自分らしさ”を追求するための土台を作る行為だ。  
+マズロー風に言えば、性的欲求が満たされないままでは、自己実現はほぼ不可能。</t>
+  </si>
+  <si>
+    <t>「モテたきゃ金銭的リスク取れ」は嘘。
+チー牛が人並に女を抱けるようになるまでは、ほぼリスクはない。
+実際に童貞捨てるまで俺が取ったリスクは
+・美容室代　7000円/月
+・服をそろえる　約7万円
+・マッチングアプリ　1万2000円
+せいぜい、こんなもん。</t>
+  </si>
+  <si>
+    <t>【脱チー牛に必要or不要な男磨き】
+【必要】
+・短期のオナ禁
+・バルクアップ
+・スキンケア
+・清潔感を洗練させる
+・ロールモデルの確立
+・美容院＆ヘアセットスキル
+・無難なファッション
+【不要】
+・長期のオナ禁
+・コールドシャワー
+・皮一枚になるまでの減量
+・ナンパ
+・メンズメイク</t>
+  </si>
+  <si>
+    <t>ち◯こを木のように勃起させる方法
+①有酸素運動
+→血流UP
+②下半身中心の筋トレ
+→テストステロン＆血流UP
+③睡眠7〜8時間
+→その日のパンプを左右する
+④シトルリン
+→パンプ感が増す
+⑤亜鉛・ビタミンD・オメガ3
+→ホルモンバランスを整える
+⑥ストレス管理
+→コルチゾールを減らす
+⑦オナ禁3〜7日</t>
+  </si>
+  <si>
+    <t>清潔感は一つでもミスったらアウト。
+※外出前に確認必須のリスト↓
+【スキンケア】
+☑睡眠食事運動の徹底
+☑保湿
+☑紫外線予防
+☑湯船につかり汗を出す
+【体毛の処理】
+☑鼻毛
+☑指毛
+☑顔そり
+☑腕毛
+☑うなじ
+【ヘアケア】
+☑ヘアオイルでパサつき抑える
+☑シャンプーを使いすぎない</t>
+  </si>
+  <si>
+    <t>情弱が引っかかる「男磨きのワナ」と「正しい努力」のやり方。
+※私は全て経験済みです。
+①小顔マッサージ
+→水分が移動しているだけなので、一時的な効果のみ。
+筋トレして肩幅を広げれば、相対的に小顔になる。
+②読書
+→目的のない読書は時間対効果が最悪。</t>
+  </si>
+  <si>
+    <t>妄想童貞オナ禁くん（20歳）の俺が本気で信じていたスーパーパワー
+・100日目で逆ナンされる
+・7日目で記憶力10倍
+・精子を貯めると筋肉がつきやすい
+・一発抜いたらテストステロン底落ち
+・オナ禁フェロモンが女を呼び寄せる
+・電車で隣に美女が座ったらオナ禁の効果</t>
+  </si>
+  <si>
+    <t>【童貞は3タイプ】
+自分の型を見極めて、正しい努力をしろ。
+①ダウナー型童貞
+→ネガティブで自信がない。いじめ・失恋・受験失敗などのトラウマ持ち。
+ 成功法： 小さな成功で自己肯定感を上げろ。筋トレが一番手っ取り早い。
+②アッパー型童貞</t>
+  </si>
+  <si>
+    <t>理想主義型の童貞について。
+「マチアプは嫌。自然に出会いたい」
+「いつか自分にふさわしい女性が現れてくれる」と理想だけ肥大化して、身動きが取れなくなるタイプ。
+舐めたこと言ってんなよ。
+俺が20歳の時に童貞卒業した相手は47歳のニューハーフだ。
+現実を見て、動き出せ。</t>
+  </si>
+  <si>
+    <t>【視野を狭めることで迷いを断つ】
+19歳の頃、自閉症チー牛だった俺はメンズコーチジョージを見まくっていた。
+散歩中、筋トレ中、食事中。
+彼の話をヘッドホンで教祖の声かのように聴きまくる日々。
+ひたすら、モテるために行動していた。
+今思うと、だいぶ狭い世界で生きてたなと思うけど、</t>
+  </si>
+  <si>
+    <t>お前がナヨナヨしている理由は、親が甘やかしてきたからだ。
+親元にいると「決断力」が育たない。
+俺がその典型で、人生の選択をほぼ母親に任せていた。
+「今日のごはん何にする？」から
+「どこの高校に進むか」まで。
+こうして、人に提案されないと動けない“モブ男”が完成する。</t>
+  </si>
+  <si>
+    <t>【弱者男性になってしまう習慣6/100】
+🚫ボソボソ喋る
+🔻解説
+原因は
+・根本的な自信のなさ
+・浅い呼吸
+・声帯の衰え
+ボソボソ喋っている内はモテない。
+その上、舐められ自信がなくなり、さらにボソボソ喋るようになるという悪循環に陥る。
+解決策は
+・男磨きで自信をつける
+・腹式呼吸を習慣化</t>
+  </si>
+  <si>
+    <t>ぶっちゃけ、プロテイン・クレアチン以外のサプリは「あったらいいな」程度。
+サプリを摂らなくてはいけないという考えは洗脳。
+長年、インフルエンサーが植え付けてきた”まやかし”なのよ。
+まず、食事を見直そう。
+そして、その食事から摂らない栄養素を補う事がサプリの役割。</t>
+  </si>
+  <si>
+    <t>空腹時の筋トレはやめよう。
+・パフォーマンス低下
+・筋分解リスクが上がる
+・血糖値が低くて集中力も落ちる
+「出勤前に筋トレしたくて、食事と消化の時間がない」という人はプロテイン・EAA飲むのもアリ。
+でも、それは仕方ない時の妥協案と思っておいてほしい。</t>
+  </si>
+  <si>
+    <t>【当たり前にやるべき口臭ケア】
+やってなければ、口からう〇この臭いがすること間違いなし。
+・フロス
+・腸活
+・歯周ポケットを意識した歯磨き
+・鼻呼吸
+・就寝時にマウステープ
+・水一日2L~4L
+・舌磨き
+・舌を上顎に付ける
+口臭に自信を持てると、声に覇気が出てくる。</t>
+  </si>
+  <si>
+    <t>「モテるために生きる」
+これは、あくまでも通過儀礼。
+だから、経験してないくせして馬鹿にするのは違う。
+また、いつまでもモテに執着するのも違う。
+前者は非モテの正当化。
+後者は30代にもなって「女を沼らせるLINE」を考えている痛いおっさんになる。
+非モテには言い訳している暇はない。</t>
+  </si>
+  <si>
+    <t>【ナヨナヨした性格は運動不足が原因】
+このメカニズムが理解できれば、いかに運動が重要かを心に刻むことが出来ます。
+🔻メカニズム
+・不安とは、危険を知らせ逃げるための警報機
+↓
+・運動不足の人は運動能力が低い。
+↓
+・運動能力が低い人は逃げるのが遅い。
+↓</t>
+  </si>
+  <si>
+    <t>童貞がモテ始めた時のサイン
+・女のボディタッチ
+・私的な質問をされる
+・物理的に近づいてくる
+・照れ笑いされる
+・平均レベルとマッチする
+・ストーリーにいいねが来る
+・相手の声が高くなる
+・目の瞳孔が開いている
+・アイコンタクトが増える</t>
+  </si>
+  <si>
+    <t>脱スマホ依存は意志力に頼ったら負け。
+なぜなら、シリコンバレーの天才たちがSNSを設計しているから。
+そんな「意志では抵抗できないドーパミン装置」がスマホなわけ。
+俺はニート時代に平均スクリーンタイム12時間のスマホ廃人だった。</t>
+  </si>
+  <si>
+    <t>スマホ新法が話題になってるけど、問題なのは時間じゃないのよ。
+・主体性を持って使う。
+or
+・脳の刺激に任せて使う。
+後者がスマホ依存症なわけ。
+・Xを5時間やってお金を稼いでいる人。
+or
+・無目的で3時間見ている人。
+後者はスクリーンタイムが少なくても、依存症である。</t>
+  </si>
+  <si>
+    <t>童貞は童貞じゃないフリをしろ。
+ハッタリをかませば、実力が追いついてくるよ。
+俺は大学入学時、彼女持ちだと嘘をつきまくった。
+結果、それっぽい振る舞いが出来るようになって、モテを攻略できたわけ。
+できる奴はハッタリをかまして、周りを動かす＆自分にプレッシャーをかける。</t>
+  </si>
+  <si>
+    <t>【目標が小さい奴は負ける】
+・「俺は細マッチョでいいや」
+→１年前と変わらずガリガリ
+・「1人の女性に好かれたい」
+→誰からも好かれない非モテ
+・「とりあえず公務員で人生安泰」
+→低給激務でコキ使われる。
+70点くらいを目指して努力している奴は、結局40点50点で終わってしまう。</t>
+  </si>
+  <si>
+    <t>【なぜAndroid＝チー牛なのか？】
+消費者行動論の視点で解説します。
+まず、人間のこだわりは以下の2つに分類される。
+①機能的価値（実利）：実際の能力・数字的スペック
+②情緒的価値（見栄・ブランド）：見た目・ステータス・第一印象
+チー牛、特にASDは①を重視する。</t>
+  </si>
+  <si>
+    <t>「1人の女性に好かれる」
+これは生物学的にありえないのよ。
+モテる奴はとことんモテて、モテない奴は全くモテない。
+これが真実。
+「学生時代、モブ男だったけどアプリを使ったらモテモテに！」なんて広告に出てくるような物語はあり得ない。
+自由恋愛は、シビアな実力主義。</t>
+  </si>
+  <si>
+    <t>「筋トレよりも食べるのが苦手」なら活動量を見直せ
+1日中歩きまくって、1レップも挙がらなくなるまで高強度の筋トレをしていたら、否が応でも食べたくなる。
+理論的には、食べるから高強度の筋トレできるが正しい
+でも、俺含めてヒョロガリ体質な人は、運動は好きだけど、食べることがマジで嫌い。</t>
+  </si>
+  <si>
+    <t>「ヒョロガリだからジム行くの恥ずかしい」
+→これ、完全に誤解。
+みんな自分の筋トレに必死で、あなたを見てる暇なんてない。
+むしろ、ジムで初心者を見ると「自宅で5分トレに騙されない賢い人だな」って思う。
+筋肉つけたいなら、
+・自宅5分トレ
+・しょぼいホームジム</t>
+  </si>
+  <si>
+    <t>結局、人は「結果」よりも「なぐさめ」がほしいだけなんだなと感じる。
+筋トレ界隈ではこれが顕著。
+「自宅で5分トレ」が爆伸びするけど、ジムで黙々とトレーニングする動画は不人気。
+某EAA野郎が人気で、ミスターオリンピアの山岸さんが伸びていない。
+これが答え。</t>
+  </si>
+  <si>
+    <t>【神サプリ VS ゴミサプリ】
+ゴミサプリに月4,000円払うなら、ジム代をケチるな
+【神サプリ】
+・プロテイン
+・クレアチン
+・プレワークアウト
+・クラスターデキストリン
+・マグネシウム
+・整腸剤
+【ゴミサプリ】
+・EAA
+・BCAA
+・HMB（き〇しん）
+・脂肪燃焼サプリ</t>
+  </si>
+  <si>
+    <t>1+1=2という真実は
+中卒が言ってようが、
+オックスフォード大卒が言ってようが変わらない。
+そこに説得力の概念はない。”
+という話。
+説得力を重要視する人は権威に弱い。
+例えば、「○○式」「△△大卒」という謳い文句や後ろ盾を見ると価値があると勘違いしてしまう。</t>
+  </si>
+  <si>
+    <t>結局、重要なのは地味なことをやり続ける能力。
+・週5の筋トレ
+・8時間睡眠
+・PCFを意識した食事
+どれも斬新ではないし、SNS映えもしない。
+でも、確実に自分を変える王道の習慣。
+逆張りをしてインプを稼ぐのが発信者としての宿命かもしれない。
+だが、俺は数字のために逆張りはしない。</t>
+  </si>
+  <si>
+    <t>【弱者男性化してしまう23の習慣】
+🔻生き方
+・他責思考
+・行動＜準備
+・男磨き陰キャ
+・自己主張しない
+・長期的快楽＜短期的快楽
+・🤓「金稼いで女を見返すやで！」
+・他人を応援（推し活、スポーツ観戦）
+🔻見た目
+・口呼吸
+・巻き肩
+・無表情
+・ヒョロガリ
+・眉毛ゲジゲジ
+・短髪ノーセット</t>
+  </si>
+  <si>
+    <t>「顔痩せ」は絶対に起こりません。
+体脂肪は“部分的”に燃焼できないからです。
+痩せる＝体全体の脂肪が減ること。
+確かに「最初に落ちる部位」「最後に落ちる部位」には個人差がありますが、顔だけ狙って脂肪を落とす方法はありません。
+顔をスッキリさせたいなら、
+①食事管理＋全身の脂肪減少</t>
+  </si>
+  <si>
+    <t>「チー牛」が流行った本当の理由。
+かつて「オタク＝チー牛」だった。
+でもオタク文化が一般化して、アニメやゲームが当たり前になった結果「童顔・無気力・モテなさそうな男」を指す言葉が消えてしまった。
+そこで現れたのが「チー牛」。</t>
+  </si>
+  <si>
+    <t>チー牛は何も考えずに身体だけ鍛えろ。
+余裕で7割の悩みは解決する。
+・男に舐められる→ヒョロガリだから
+・女にモテない→ヒョロガリだから
+・自信がない→ヒョロガリだから
+・服が似合わない→ヒョロガリだから
+・コミュ障→ヒョロガリだから
+・鬱っぽい→テストステロン不足</t>
+  </si>
+  <si>
+    <t>トレ後の食事と同様にトレ前の食事が重要。
+「筋トレ後にすぐタンパク質を取らないと筋分解されちゃう🙀」
+この強迫観念で、トレ後の食事は完璧な人が多い。
+でも、足りていないのはトレ前の食事だ。
+特に炭水化物は筋トレの持続力と出力を引き上げてくれる。</t>
+  </si>
+  <si>
+    <t>「チー牛家庭」の問題点。
+・食事から教育方針まで、すべて母親が決める
+・母親の地位が高く、父親は空気。
+一見サポート的に見えるけど、問題はここから。
+就職など「大きな決断」が迫った時、母親は逃げる。
+はしごを外され、決断力を育ててこなかったチー牛はあっという間に迷子になる。</t>
+  </si>
+  <si>
+    <t>俺がアスペを自覚する前に犯していた恋愛上のミス
+・会話＝議論
+・自分語り＝コミュ力
+・無表情＝クール
+・話し方＜話す内容
+・外見＜性格
+・共感＜事実の陳列
+・相手への興味0
+・IQ＝150　EQ＝0
+対処法は、まず自分を理解する事。
+理解すると</t>
+  </si>
+  <si>
+    <t>オナ禁を少し擁護すると
+・短期的にテストステロンが向上
+・衝動を制御し自己規律が身につく
+・勃起力の向上
+といった恩恵を受けることが出来る。
+確かに長期でやるのは無意味。</t>
+  </si>
+  <si>
+    <t>男磨きコンテンツに群がる層は「今まで男磨きが当たり前ではなかった弱者」しかいない。
+幼少期からスポーツや身だしなみが習慣化している層は
+わざわざ「男磨き」という概念に頼らなくても自然にやっている。
+この世に性別は2つしかないから男磨きなんて当たり前の事。呼吸のようにやれ。</t>
+  </si>
+  <si>
+    <t>「まず知識を得てから」という癖がある人は成長が遅い。勉強＜行動な理由は「自分事にするため」です。
+行動しないと自分ごとにならずインプットの質も落ちる。
+・読書→行動❌
+行動する→行き詰る→課題解決のために読書⭕
+・SNSマーケを学び発信❌
+発信をしつつSNSマーケを学んでいく⭕</t>
+  </si>
+  <si>
+    <t>清潔感＝モテは間違い。
+理由を端的に言えば、マイナスが0になっただけだから。
+あなたがガチのイケメンじゃない限り、清潔感を出してやっと普通の男として見られるレベル。
+清潔感を当たり前にクリアした上で、あなたのアイデンティティやステータスとなる金、顔、筋肉etc.を磨いていく。</t>
+  </si>
+  <si>
+    <t>「デブは普通に生きていたらならない」と言うが、むしろ普通に生きているからこそデブになる。
+人類がサバンナで暮らしていた時代、食料は常に不足し、飢餓との戦いだった。
+そんな環境で生き延びたのは「目の前にカロリーがあるならすぐに摂取する個体」だった。</t>
+  </si>
+  <si>
+    <t>睡眠不足の日の対処法
+・朝散歩
+・有酸素30分
+・朝にコーヒー
+・筋トレは控える
+・夜にメラトニンサプリ
+・起床後にカーテンを開ける
+・午後はカフェインを控える
+本当に睡眠不足の時はジムをサボってもいい。
+無理やりカフェインで覚醒させてもクソトレにしかならない。</t>
+  </si>
+  <si>
+    <t>僕は毎朝コールドシャワーを浴びて10分間瞑想をします！そしてジャーナルにToDoと目標を書きます。
+朝飯は抜きます。
+サーモンは生物濃縮でマイクロプラスティックが含まれているため、週に一回しか食べません。</t>
+  </si>
+  <si>
+    <t>食べても食べても体重が増えない人は、食べる量に“波”があります。
+例えば、あなたのメンテナンスカロリーが2800kcalだとしましょう。
+ある日ドカ食いして3800kcal（＋1000kcalの余剰）を摂っても、翌日にお腹を壊して1800kcalしか食べられなければ、2日間の平均はちょうど2800kcal。</t>
+  </si>
+  <si>
+    <t>仮にあなたが
+「筋肉で女の子を沼らせたい」
+「ゴリマッチョにはなりたくない」
+と思っていても筋トレはボディビルダーから学ぶべきです。
+なぜなら、彼らは「筋肥大」という明確な目的に人生を懸けている、いわば“筋肉のプロフェッショナル”だからです。</t>
+  </si>
+  <si>
+    <t>巷の「モテるための筋トレ」はユニセフのCMに出てくるアフガキ体型になる筋トレです。
+あなた程度の筋肉量で体脂肪率を10%以下にする必要はありません。
+バルクアップをして高重量を持ちましょう。
+単純に体重が重い方が高重量が扱いやすいので。</t>
   </si>
 </sst>
 </file>
@@ -34140,7 +36335,7 @@
         <ns0:v>474</ns0:v>
       </ns0:c>
       <ns0:c r="B238" t="s" s="0">
-        <ns0:v>4129</ns0:v>
+        <ns0:v>4679</ns0:v>
       </ns0:c>
       <ns0:c r="C238">
         <ns0:v>0</ns0:v>
@@ -34174,7 +36369,7 @@
         <ns0:v>478</ns0:v>
       </ns0:c>
       <ns0:c r="B240" t="s" s="0">
-        <ns0:v>4130</ns0:v>
+        <ns0:v>4680</ns0:v>
       </ns0:c>
       <ns0:c r="C240">
         <ns0:v>5</ns0:v>
@@ -34327,7 +36522,7 @@
         <ns0:v>496</ns0:v>
       </ns0:c>
       <ns0:c r="B249" t="s" s="0">
-        <ns0:v>4131</ns0:v>
+        <ns0:v>4681</ns0:v>
       </ns0:c>
       <ns0:c r="C249">
         <ns0:v>3</ns0:v>
@@ -34361,7 +36556,7 @@
         <ns0:v>500</ns0:v>
       </ns0:c>
       <ns0:c r="B251" t="s" s="0">
-        <ns0:v>4132</ns0:v>
+        <ns0:v>4682</ns0:v>
       </ns0:c>
       <ns0:c r="C251">
         <ns0:v>7</ns0:v>
@@ -34378,7 +36573,7 @@
         <ns0:v>502</ns0:v>
       </ns0:c>
       <ns0:c r="B252" t="s" s="0">
-        <ns0:v>4133</ns0:v>
+        <ns0:v>4683</ns0:v>
       </ns0:c>
       <ns0:c r="C252">
         <ns0:v>2</ns0:v>
@@ -34395,7 +36590,7 @@
         <ns0:v>504</ns0:v>
       </ns0:c>
       <ns0:c r="B253" t="s" s="0">
-        <ns0:v>4134</ns0:v>
+        <ns0:v>4684</ns0:v>
       </ns0:c>
       <ns0:c r="C253">
         <ns0:v>1</ns0:v>
@@ -34429,7 +36624,7 @@
         <ns0:v>508</ns0:v>
       </ns0:c>
       <ns0:c r="B255" t="s" s="0">
-        <ns0:v>4135</ns0:v>
+        <ns0:v>4685</ns0:v>
       </ns0:c>
       <ns0:c r="C255">
         <ns0:v>10</ns0:v>
@@ -34497,7 +36692,7 @@
         <ns0:v>516</ns0:v>
       </ns0:c>
       <ns0:c r="B259" t="s" s="0">
-        <ns0:v>4136</ns0:v>
+        <ns0:v>4686</ns0:v>
       </ns0:c>
       <ns0:c r="C259">
         <ns0:v>2</ns0:v>
@@ -34582,7 +36777,7 @@
         <ns0:v>526</ns0:v>
       </ns0:c>
       <ns0:c r="B264" t="s" s="0">
-        <ns0:v>4137</ns0:v>
+        <ns0:v>4687</ns0:v>
       </ns0:c>
       <ns0:c r="C264">
         <ns0:v>2</ns0:v>
@@ -34599,7 +36794,7 @@
         <ns0:v>528</ns0:v>
       </ns0:c>
       <ns0:c r="B265" t="s" s="0">
-        <ns0:v>4138</ns0:v>
+        <ns0:v>4688</ns0:v>
       </ns0:c>
       <ns0:c r="C265">
         <ns0:v>2</ns0:v>
@@ -34667,7 +36862,7 @@
         <ns0:v>536</ns0:v>
       </ns0:c>
       <ns0:c r="B269" t="s" s="0">
-        <ns0:v>4139</ns0:v>
+        <ns0:v>4689</ns0:v>
       </ns0:c>
       <ns0:c r="C269">
         <ns0:v>0</ns0:v>
@@ -34718,7 +36913,7 @@
         <ns0:v>542</ns0:v>
       </ns0:c>
       <ns0:c r="B272" t="s" s="0">
-        <ns0:v>4140</ns0:v>
+        <ns0:v>4690</ns0:v>
       </ns0:c>
       <ns0:c r="C272">
         <ns0:v>13</ns0:v>
@@ -34735,7 +36930,7 @@
         <ns0:v>544</ns0:v>
       </ns0:c>
       <ns0:c r="B273" t="s" s="0">
-        <ns0:v>4141</ns0:v>
+        <ns0:v>4691</ns0:v>
       </ns0:c>
       <ns0:c r="C273">
         <ns0:v>2</ns0:v>
@@ -34803,7 +36998,7 @@
         <ns0:v>552</ns0:v>
       </ns0:c>
       <ns0:c r="B277" t="s" s="0">
-        <ns0:v>4142</ns0:v>
+        <ns0:v>4692</ns0:v>
       </ns0:c>
       <ns0:c r="C277">
         <ns0:v>14</ns0:v>
@@ -34837,7 +37032,7 @@
         <ns0:v>556</ns0:v>
       </ns0:c>
       <ns0:c r="B279" t="s" s="0">
-        <ns0:v>4143</ns0:v>
+        <ns0:v>4693</ns0:v>
       </ns0:c>
       <ns0:c r="C279">
         <ns0:v>4</ns0:v>
@@ -35007,7 +37202,7 @@
         <ns0:v>575</ns0:v>
       </ns0:c>
       <ns0:c r="B289" t="s" s="0">
-        <ns0:v>4144</ns0:v>
+        <ns0:v>4694</ns0:v>
       </ns0:c>
       <ns0:c r="C289">
         <ns0:v>0</ns0:v>
@@ -35024,7 +37219,7 @@
         <ns0:v>577</ns0:v>
       </ns0:c>
       <ns0:c r="B290" t="s" s="0">
-        <ns0:v>4145</ns0:v>
+        <ns0:v>4695</ns0:v>
       </ns0:c>
       <ns0:c r="C290">
         <ns0:v>1</ns0:v>
@@ -35041,7 +37236,7 @@
         <ns0:v>579</ns0:v>
       </ns0:c>
       <ns0:c r="B291" t="s" s="0">
-        <ns0:v>4146</ns0:v>
+        <ns0:v>4696</ns0:v>
       </ns0:c>
       <ns0:c r="C291">
         <ns0:v>2</ns0:v>
@@ -35092,7 +37287,7 @@
         <ns0:v>585</ns0:v>
       </ns0:c>
       <ns0:c r="B294" t="s" s="0">
-        <ns0:v>4147</ns0:v>
+        <ns0:v>4697</ns0:v>
       </ns0:c>
       <ns0:c r="C294">
         <ns0:v>2</ns0:v>
@@ -35143,7 +37338,7 @@
         <ns0:v>591</ns0:v>
       </ns0:c>
       <ns0:c r="B297" t="s" s="0">
-        <ns0:v>4148</ns0:v>
+        <ns0:v>4698</ns0:v>
       </ns0:c>
       <ns0:c r="C297">
         <ns0:v>1</ns0:v>
@@ -35160,7 +37355,7 @@
         <ns0:v>593</ns0:v>
       </ns0:c>
       <ns0:c r="B298" t="s" s="0">
-        <ns0:v>4149</ns0:v>
+        <ns0:v>4699</ns0:v>
       </ns0:c>
       <ns0:c r="C298">
         <ns0:v>4</ns0:v>
@@ -35211,7 +37406,7 @@
         <ns0:v>599</ns0:v>
       </ns0:c>
       <ns0:c r="B301" t="s" s="0">
-        <ns0:v>4150</ns0:v>
+        <ns0:v>4700</ns0:v>
       </ns0:c>
       <ns0:c r="C301">
         <ns0:v>6</ns0:v>
@@ -35313,7 +37508,7 @@
         <ns0:v>611</ns0:v>
       </ns0:c>
       <ns0:c r="B307" t="s" s="0">
-        <ns0:v>4151</ns0:v>
+        <ns0:v>4701</ns0:v>
       </ns0:c>
       <ns0:c r="C307">
         <ns0:v>0</ns0:v>
@@ -35432,7 +37627,7 @@
         <ns0:v>625</ns0:v>
       </ns0:c>
       <ns0:c r="B314" t="s" s="0">
-        <ns0:v>4152</ns0:v>
+        <ns0:v>4702</ns0:v>
       </ns0:c>
       <ns0:c r="C314">
         <ns0:v>2</ns0:v>
@@ -35449,7 +37644,7 @@
         <ns0:v>627</ns0:v>
       </ns0:c>
       <ns0:c r="B315" t="s" s="0">
-        <ns0:v>4153</ns0:v>
+        <ns0:v>4703</ns0:v>
       </ns0:c>
       <ns0:c r="C315">
         <ns0:v>0</ns0:v>
@@ -35466,7 +37661,7 @@
         <ns0:v>629</ns0:v>
       </ns0:c>
       <ns0:c r="B316" t="s" s="0">
-        <ns0:v>4154</ns0:v>
+        <ns0:v>4704</ns0:v>
       </ns0:c>
       <ns0:c r="C316">
         <ns0:v>1</ns0:v>
@@ -35534,7 +37729,7 @@
         <ns0:v>637</ns0:v>
       </ns0:c>
       <ns0:c r="B320" t="s" s="0">
-        <ns0:v>4155</ns0:v>
+        <ns0:v>4705</ns0:v>
       </ns0:c>
       <ns0:c r="C320">
         <ns0:v>3</ns0:v>
@@ -35551,7 +37746,7 @@
         <ns0:v>639</ns0:v>
       </ns0:c>
       <ns0:c r="B321" t="s" s="0">
-        <ns0:v>4156</ns0:v>
+        <ns0:v>4706</ns0:v>
       </ns0:c>
       <ns0:c r="C321">
         <ns0:v>0</ns0:v>
@@ -35585,7 +37780,7 @@
         <ns0:v>643</ns0:v>
       </ns0:c>
       <ns0:c r="B323" t="s" s="0">
-        <ns0:v>4157</ns0:v>
+        <ns0:v>4707</ns0:v>
       </ns0:c>
       <ns0:c r="C323">
         <ns0:v>1</ns0:v>
@@ -35636,7 +37831,7 @@
         <ns0:v>649</ns0:v>
       </ns0:c>
       <ns0:c r="B326" t="s" s="0">
-        <ns0:v>4158</ns0:v>
+        <ns0:v>4708</ns0:v>
       </ns0:c>
       <ns0:c r="C326">
         <ns0:v>0</ns0:v>
@@ -35653,7 +37848,7 @@
         <ns0:v>651</ns0:v>
       </ns0:c>
       <ns0:c r="B327" t="s" s="0">
-        <ns0:v>4159</ns0:v>
+        <ns0:v>4709</ns0:v>
       </ns0:c>
       <ns0:c r="C327">
         <ns0:v>2</ns0:v>
@@ -35772,7 +37967,7 @@
         <ns0:v>665</ns0:v>
       </ns0:c>
       <ns0:c r="B334" t="s" s="0">
-        <ns0:v>4160</ns0:v>
+        <ns0:v>4710</ns0:v>
       </ns0:c>
       <ns0:c r="C334">
         <ns0:v>0</ns0:v>
@@ -35789,7 +37984,7 @@
         <ns0:v>667</ns0:v>
       </ns0:c>
       <ns0:c r="B335" t="s" s="0">
-        <ns0:v>4161</ns0:v>
+        <ns0:v>4711</ns0:v>
       </ns0:c>
       <ns0:c r="C335">
         <ns0:v>1</ns0:v>
@@ -36027,7 +38222,7 @@
         <ns0:v>695</ns0:v>
       </ns0:c>
       <ns0:c r="B349" t="s" s="0">
-        <ns0:v>4162</ns0:v>
+        <ns0:v>4712</ns0:v>
       </ns0:c>
       <ns0:c r="C349">
         <ns0:v>2</ns0:v>
@@ -36044,7 +38239,7 @@
         <ns0:v>697</ns0:v>
       </ns0:c>
       <ns0:c r="B350" t="s" s="0">
-        <ns0:v>4163</ns0:v>
+        <ns0:v>4713</ns0:v>
       </ns0:c>
       <ns0:c r="C350">
         <ns0:v>4</ns0:v>
@@ -36095,7 +38290,7 @@
         <ns0:v>703</ns0:v>
       </ns0:c>
       <ns0:c r="B353" t="s" s="0">
-        <ns0:v>4164</ns0:v>
+        <ns0:v>4714</ns0:v>
       </ns0:c>
       <ns0:c r="C353">
         <ns0:v>3</ns0:v>
@@ -36180,7 +38375,7 @@
         <ns0:v>713</ns0:v>
       </ns0:c>
       <ns0:c r="B358" t="s" s="0">
-        <ns0:v>4165</ns0:v>
+        <ns0:v>4715</ns0:v>
       </ns0:c>
       <ns0:c r="C358">
         <ns0:v>1</ns0:v>
@@ -36265,7 +38460,7 @@
         <ns0:v>723</ns0:v>
       </ns0:c>
       <ns0:c r="B363" t="s" s="0">
-        <ns0:v>4166</ns0:v>
+        <ns0:v>4716</ns0:v>
       </ns0:c>
       <ns0:c r="C363">
         <ns0:v>0</ns0:v>
@@ -36282,7 +38477,7 @@
         <ns0:v>725</ns0:v>
       </ns0:c>
       <ns0:c r="B364" t="s" s="0">
-        <ns0:v>4167</ns0:v>
+        <ns0:v>4717</ns0:v>
       </ns0:c>
       <ns0:c r="C364">
         <ns0:v>0</ns0:v>
@@ -36316,7 +38511,7 @@
         <ns0:v>729</ns0:v>
       </ns0:c>
       <ns0:c r="B366" t="s" s="0">
-        <ns0:v>4168</ns0:v>
+        <ns0:v>4718</ns0:v>
       </ns0:c>
       <ns0:c r="C366">
         <ns0:v>6</ns0:v>
@@ -36384,7 +38579,7 @@
         <ns0:v>737</ns0:v>
       </ns0:c>
       <ns0:c r="B370" t="s" s="0">
-        <ns0:v>4169</ns0:v>
+        <ns0:v>4719</ns0:v>
       </ns0:c>
       <ns0:c r="C370">
         <ns0:v>4</ns0:v>
@@ -36452,7 +38647,7 @@
         <ns0:v>745</ns0:v>
       </ns0:c>
       <ns0:c r="B374" t="s" s="0">
-        <ns0:v>4170</ns0:v>
+        <ns0:v>4720</ns0:v>
       </ns0:c>
       <ns0:c r="C374">
         <ns0:v>3</ns0:v>
@@ -36503,7 +38698,7 @@
         <ns0:v>751</ns0:v>
       </ns0:c>
       <ns0:c r="B377" t="s" s="0">
-        <ns0:v>4171</ns0:v>
+        <ns0:v>4721</ns0:v>
       </ns0:c>
       <ns0:c r="C377">
         <ns0:v>1</ns0:v>
@@ -36537,7 +38732,7 @@
         <ns0:v>755</ns0:v>
       </ns0:c>
       <ns0:c r="B379" t="s" s="0">
-        <ns0:v>4172</ns0:v>
+        <ns0:v>4722</ns0:v>
       </ns0:c>
       <ns0:c r="C379">
         <ns0:v>1</ns0:v>
@@ -36588,7 +38783,7 @@
         <ns0:v>761</ns0:v>
       </ns0:c>
       <ns0:c r="B382" t="s" s="0">
-        <ns0:v>4173</ns0:v>
+        <ns0:v>4723</ns0:v>
       </ns0:c>
       <ns0:c r="C382">
         <ns0:v>0</ns0:v>
@@ -36605,7 +38800,7 @@
         <ns0:v>763</ns0:v>
       </ns0:c>
       <ns0:c r="B383" t="s" s="0">
-        <ns0:v>4174</ns0:v>
+        <ns0:v>4724</ns0:v>
       </ns0:c>
       <ns0:c r="C383">
         <ns0:v>0</ns0:v>
@@ -36622,7 +38817,7 @@
         <ns0:v>765</ns0:v>
       </ns0:c>
       <ns0:c r="B384" t="s" s="0">
-        <ns0:v>4175</ns0:v>
+        <ns0:v>4725</ns0:v>
       </ns0:c>
       <ns0:c r="C384">
         <ns0:v>0</ns0:v>
@@ -36656,7 +38851,7 @@
         <ns0:v>769</ns0:v>
       </ns0:c>
       <ns0:c r="B386" t="s" s="0">
-        <ns0:v>4176</ns0:v>
+        <ns0:v>4726</ns0:v>
       </ns0:c>
       <ns0:c r="C386">
         <ns0:v>3</ns0:v>
@@ -36741,7 +38936,7 @@
         <ns0:v>779</ns0:v>
       </ns0:c>
       <ns0:c r="B391" t="s" s="0">
-        <ns0:v>4177</ns0:v>
+        <ns0:v>4675</ns0:v>
       </ns0:c>
       <ns0:c r="C391">
         <ns0:v>145</ns0:v>
@@ -36792,7 +38987,7 @@
         <ns0:v>785</ns0:v>
       </ns0:c>
       <ns0:c r="B394" t="s" s="0">
-        <ns0:v>4178</ns0:v>
+        <ns0:v>4727</ns0:v>
       </ns0:c>
       <ns0:c r="C394">
         <ns0:v>0</ns0:v>
@@ -36809,7 +39004,7 @@
         <ns0:v>787</ns0:v>
       </ns0:c>
       <ns0:c r="B395" t="s" s="0">
-        <ns0:v>4179</ns0:v>
+        <ns0:v>4728</ns0:v>
       </ns0:c>
       <ns0:c r="C395">
         <ns0:v>2</ns0:v>
@@ -36894,7 +39089,7 @@
         <ns0:v>796</ns0:v>
       </ns0:c>
       <ns0:c r="B400" t="s" s="0">
-        <ns0:v>4180</ns0:v>
+        <ns0:v>4729</ns0:v>
       </ns0:c>
       <ns0:c r="C400">
         <ns0:v>6</ns0:v>
@@ -36962,7 +39157,7 @@
         <ns0:v>804</ns0:v>
       </ns0:c>
       <ns0:c r="B404" t="s" s="0">
-        <ns0:v>4181</ns0:v>
+        <ns0:v>4730</ns0:v>
       </ns0:c>
       <ns0:c r="C404">
         <ns0:v>5</ns0:v>
@@ -37013,7 +39208,7 @@
         <ns0:v>810</ns0:v>
       </ns0:c>
       <ns0:c r="B407" t="s" s="0">
-        <ns0:v>4182</ns0:v>
+        <ns0:v>4731</ns0:v>
       </ns0:c>
       <ns0:c r="C407">
         <ns0:v>3</ns0:v>
@@ -37064,7 +39259,7 @@
         <ns0:v>816</ns0:v>
       </ns0:c>
       <ns0:c r="B410" t="s" s="0">
-        <ns0:v>4183</ns0:v>
+        <ns0:v>4732</ns0:v>
       </ns0:c>
       <ns0:c r="C410">
         <ns0:v>7</ns0:v>
@@ -37081,7 +39276,7 @@
         <ns0:v>818</ns0:v>
       </ns0:c>
       <ns0:c r="B411" t="s" s="0">
-        <ns0:v>4184</ns0:v>
+        <ns0:v>4733</ns0:v>
       </ns0:c>
       <ns0:c r="C411">
         <ns0:v>1</ns0:v>
@@ -37115,7 +39310,7 @@
         <ns0:v>822</ns0:v>
       </ns0:c>
       <ns0:c r="B413" t="s" s="0">
-        <ns0:v>4185</ns0:v>
+        <ns0:v>4734</ns0:v>
       </ns0:c>
       <ns0:c r="C413">
         <ns0:v>3</ns0:v>
@@ -37132,7 +39327,7 @@
         <ns0:v>824</ns0:v>
       </ns0:c>
       <ns0:c r="B414" t="s" s="0">
-        <ns0:v>4186</ns0:v>
+        <ns0:v>4735</ns0:v>
       </ns0:c>
       <ns0:c r="C414">
         <ns0:v>0</ns0:v>
@@ -37234,7 +39429,7 @@
         <ns0:v>836</ns0:v>
       </ns0:c>
       <ns0:c r="B420" t="s" s="0">
-        <ns0:v>4187</ns0:v>
+        <ns0:v>4736</ns0:v>
       </ns0:c>
       <ns0:c r="C420">
         <ns0:v>0</ns0:v>
@@ -37251,7 +39446,7 @@
         <ns0:v>838</ns0:v>
       </ns0:c>
       <ns0:c r="B421" t="s" s="0">
-        <ns0:v>4188</ns0:v>
+        <ns0:v>4737</ns0:v>
       </ns0:c>
       <ns0:c r="C421">
         <ns0:v>0</ns0:v>
@@ -37302,7 +39497,7 @@
         <ns0:v>844</ns0:v>
       </ns0:c>
       <ns0:c r="B424" t="s" s="0">
-        <ns0:v>4189</ns0:v>
+        <ns0:v>4738</ns0:v>
       </ns0:c>
       <ns0:c r="C424">
         <ns0:v>0</ns0:v>
@@ -37336,7 +39531,7 @@
         <ns0:v>848</ns0:v>
       </ns0:c>
       <ns0:c r="B426" t="s" s="0">
-        <ns0:v>4190</ns0:v>
+        <ns0:v>4739</ns0:v>
       </ns0:c>
       <ns0:c r="C426">
         <ns0:v>1</ns0:v>
@@ -37353,7 +39548,7 @@
         <ns0:v>850</ns0:v>
       </ns0:c>
       <ns0:c r="B427" t="s" s="0">
-        <ns0:v>4191</ns0:v>
+        <ns0:v>4740</ns0:v>
       </ns0:c>
       <ns0:c r="C427">
         <ns0:v>0</ns0:v>
@@ -37370,7 +39565,7 @@
         <ns0:v>852</ns0:v>
       </ns0:c>
       <ns0:c r="B428" t="s" s="0">
-        <ns0:v>4192</ns0:v>
+        <ns0:v>4741</ns0:v>
       </ns0:c>
       <ns0:c r="C428">
         <ns0:v>2</ns0:v>
@@ -37387,7 +39582,7 @@
         <ns0:v>854</ns0:v>
       </ns0:c>
       <ns0:c r="B429" t="s" s="0">
-        <ns0:v>4193</ns0:v>
+        <ns0:v>4742</ns0:v>
       </ns0:c>
       <ns0:c r="C429">
         <ns0:v>4</ns0:v>
@@ -37472,7 +39667,7 @@
         <ns0:v>864</ns0:v>
       </ns0:c>
       <ns0:c r="B434" t="s" s="0">
-        <ns0:v>4194</ns0:v>
+        <ns0:v>4743</ns0:v>
       </ns0:c>
       <ns0:c r="C434">
         <ns0:v>0</ns0:v>
@@ -37506,7 +39701,7 @@
         <ns0:v>868</ns0:v>
       </ns0:c>
       <ns0:c r="B436" t="s" s="0">
-        <ns0:v>4195</ns0:v>
+        <ns0:v>4744</ns0:v>
       </ns0:c>
       <ns0:c r="C436">
         <ns0:v>0</ns0:v>
@@ -37574,7 +39769,7 @@
         <ns0:v>876</ns0:v>
       </ns0:c>
       <ns0:c r="B440" t="s" s="0">
-        <ns0:v>4196</ns0:v>
+        <ns0:v>4745</ns0:v>
       </ns0:c>
       <ns0:c r="C440">
         <ns0:v>1</ns0:v>
@@ -37608,7 +39803,7 @@
         <ns0:v>880</ns0:v>
       </ns0:c>
       <ns0:c r="B442" t="s" s="0">
-        <ns0:v>4197</ns0:v>
+        <ns0:v>4746</ns0:v>
       </ns0:c>
       <ns0:c r="C442">
         <ns0:v>0</ns0:v>
@@ -37642,7 +39837,7 @@
         <ns0:v>884</ns0:v>
       </ns0:c>
       <ns0:c r="B444" t="s" s="0">
-        <ns0:v>4198</ns0:v>
+        <ns0:v>4747</ns0:v>
       </ns0:c>
       <ns0:c r="C444">
         <ns0:v>1</ns0:v>
@@ -37659,7 +39854,7 @@
         <ns0:v>886</ns0:v>
       </ns0:c>
       <ns0:c r="B445" t="s" s="0">
-        <ns0:v>4199</ns0:v>
+        <ns0:v>4748</ns0:v>
       </ns0:c>
       <ns0:c r="C445">
         <ns0:v>0</ns0:v>
@@ -37693,7 +39888,7 @@
         <ns0:v>890</ns0:v>
       </ns0:c>
       <ns0:c r="B447" t="s" s="0">
-        <ns0:v>4200</ns0:v>
+        <ns0:v>4749</ns0:v>
       </ns0:c>
       <ns0:c r="C447">
         <ns0:v>0</ns0:v>
@@ -37761,7 +39956,7 @@
         <ns0:v>898</ns0:v>
       </ns0:c>
       <ns0:c r="B451" t="s" s="0">
-        <ns0:v>4201</ns0:v>
+        <ns0:v>4750</ns0:v>
       </ns0:c>
       <ns0:c r="C451">
         <ns0:v>3</ns0:v>
@@ -37778,7 +39973,7 @@
         <ns0:v>900</ns0:v>
       </ns0:c>
       <ns0:c r="B452" t="s" s="0">
-        <ns0:v>4202</ns0:v>
+        <ns0:v>4751</ns0:v>
       </ns0:c>
       <ns0:c r="C452">
         <ns0:v>0</ns0:v>
@@ -37812,7 +40007,7 @@
         <ns0:v>904</ns0:v>
       </ns0:c>
       <ns0:c r="B454" t="s" s="0">
-        <ns0:v>4203</ns0:v>
+        <ns0:v>4752</ns0:v>
       </ns0:c>
       <ns0:c r="C454">
         <ns0:v>2</ns0:v>
@@ -37880,7 +40075,7 @@
         <ns0:v>912</ns0:v>
       </ns0:c>
       <ns0:c r="B458" t="s" s="0">
-        <ns0:v>4204</ns0:v>
+        <ns0:v>4753</ns0:v>
       </ns0:c>
       <ns0:c r="C458">
         <ns0:v>0</ns0:v>
@@ -37999,7 +40194,7 @@
         <ns0:v>926</ns0:v>
       </ns0:c>
       <ns0:c r="B465" t="s" s="0">
-        <ns0:v>4205</ns0:v>
+        <ns0:v>4754</ns0:v>
       </ns0:c>
       <ns0:c r="C465">
         <ns0:v>2</ns0:v>
@@ -38016,7 +40211,7 @@
         <ns0:v>928</ns0:v>
       </ns0:c>
       <ns0:c r="B466" t="s" s="0">
-        <ns0:v>4206</ns0:v>
+        <ns0:v>4755</ns0:v>
       </ns0:c>
       <ns0:c r="C466">
         <ns0:v>1</ns0:v>
@@ -38135,7 +40330,7 @@
         <ns0:v>941</ns0:v>
       </ns0:c>
       <ns0:c r="B473" t="s" s="0">
-        <ns0:v>4207</ns0:v>
+        <ns0:v>4756</ns0:v>
       </ns0:c>
       <ns0:c r="C473">
         <ns0:v>1</ns0:v>
@@ -38169,7 +40364,7 @@
         <ns0:v>945</ns0:v>
       </ns0:c>
       <ns0:c r="B475" t="s" s="0">
-        <ns0:v>4208</ns0:v>
+        <ns0:v>4757</ns0:v>
       </ns0:c>
       <ns0:c r="C475">
         <ns0:v>0</ns0:v>
@@ -38186,7 +40381,7 @@
         <ns0:v>947</ns0:v>
       </ns0:c>
       <ns0:c r="B476" t="s" s="0">
-        <ns0:v>4209</ns0:v>
+        <ns0:v>4758</ns0:v>
       </ns0:c>
       <ns0:c r="C476">
         <ns0:v>0</ns0:v>
@@ -38220,7 +40415,7 @@
         <ns0:v>951</ns0:v>
       </ns0:c>
       <ns0:c r="B478" t="s" s="0">
-        <ns0:v>4210</ns0:v>
+        <ns0:v>4759</ns0:v>
       </ns0:c>
       <ns0:c r="C478">
         <ns0:v>0</ns0:v>
@@ -38322,7 +40517,7 @@
         <ns0:v>963</ns0:v>
       </ns0:c>
       <ns0:c r="B484" t="s" s="0">
-        <ns0:v>4211</ns0:v>
+        <ns0:v>4760</ns0:v>
       </ns0:c>
       <ns0:c r="C484">
         <ns0:v>5</ns0:v>
@@ -38373,7 +40568,7 @@
         <ns0:v>969</ns0:v>
       </ns0:c>
       <ns0:c r="B487" t="s" s="0">
-        <ns0:v>4212</ns0:v>
+        <ns0:v>4761</ns0:v>
       </ns0:c>
       <ns0:c r="C487">
         <ns0:v>2</ns0:v>
@@ -38424,7 +40619,7 @@
         <ns0:v>975</ns0:v>
       </ns0:c>
       <ns0:c r="B490" t="s" s="0">
-        <ns0:v>4213</ns0:v>
+        <ns0:v>4762</ns0:v>
       </ns0:c>
       <ns0:c r="C490">
         <ns0:v>2</ns0:v>
@@ -38458,7 +40653,7 @@
         <ns0:v>979</ns0:v>
       </ns0:c>
       <ns0:c r="B492" t="s" s="0">
-        <ns0:v>4214</ns0:v>
+        <ns0:v>4763</ns0:v>
       </ns0:c>
       <ns0:c r="C492">
         <ns0:v>1</ns0:v>
@@ -38475,7 +40670,7 @@
         <ns0:v>981</ns0:v>
       </ns0:c>
       <ns0:c r="B493" t="s" s="0">
-        <ns0:v>4215</ns0:v>
+        <ns0:v>4764</ns0:v>
       </ns0:c>
       <ns0:c r="C493">
         <ns0:v>3</ns0:v>
@@ -38543,7 +40738,7 @@
         <ns0:v>989</ns0:v>
       </ns0:c>
       <ns0:c r="B497" t="s" s="0">
-        <ns0:v>4216</ns0:v>
+        <ns0:v>4765</ns0:v>
       </ns0:c>
       <ns0:c r="C497">
         <ns0:v>1</ns0:v>
@@ -38560,7 +40755,7 @@
         <ns0:v>991</ns0:v>
       </ns0:c>
       <ns0:c r="B498" t="s" s="0">
-        <ns0:v>4217</ns0:v>
+        <ns0:v>4766</ns0:v>
       </ns0:c>
       <ns0:c r="C498">
         <ns0:v>0</ns0:v>
@@ -38577,7 +40772,7 @@
         <ns0:v>993</ns0:v>
       </ns0:c>
       <ns0:c r="B499" t="s" s="0">
-        <ns0:v>4218</ns0:v>
+        <ns0:v>4767</ns0:v>
       </ns0:c>
       <ns0:c r="C499">
         <ns0:v>0</ns0:v>
@@ -38594,7 +40789,7 @@
         <ns0:v>995</ns0:v>
       </ns0:c>
       <ns0:c r="B500" t="s" s="0">
-        <ns0:v>4219</ns0:v>
+        <ns0:v>4768</ns0:v>
       </ns0:c>
       <ns0:c r="C500">
         <ns0:v>0</ns0:v>
@@ -38611,7 +40806,7 @@
         <ns0:v>997</ns0:v>
       </ns0:c>
       <ns0:c r="B501" t="s" s="0">
-        <ns0:v>4220</ns0:v>
+        <ns0:v>4769</ns0:v>
       </ns0:c>
       <ns0:c r="C501">
         <ns0:v>0</ns0:v>
@@ -38628,7 +40823,7 @@
         <ns0:v>999</ns0:v>
       </ns0:c>
       <ns0:c r="B502" t="s" s="0">
-        <ns0:v>4221</ns0:v>
+        <ns0:v>4770</ns0:v>
       </ns0:c>
       <ns0:c r="C502">
         <ns0:v>0</ns0:v>
@@ -38730,7 +40925,7 @@
         <ns0:v>1011</ns0:v>
       </ns0:c>
       <ns0:c r="B508" t="s" s="0">
-        <ns0:v>4222</ns0:v>
+        <ns0:v>4771</ns0:v>
       </ns0:c>
       <ns0:c r="C508">
         <ns0:v>0</ns0:v>
@@ -38798,7 +40993,7 @@
         <ns0:v>1019</ns0:v>
       </ns0:c>
       <ns0:c r="B512" t="s" s="0">
-        <ns0:v>4223</ns0:v>
+        <ns0:v>4772</ns0:v>
       </ns0:c>
       <ns0:c r="C512">
         <ns0:v>0</ns0:v>
@@ -38832,7 +41027,7 @@
         <ns0:v>1023</ns0:v>
       </ns0:c>
       <ns0:c r="B514" t="s" s="0">
-        <ns0:v>4224</ns0:v>
+        <ns0:v>4773</ns0:v>
       </ns0:c>
       <ns0:c r="C514">
         <ns0:v>4</ns0:v>
@@ -38866,7 +41061,7 @@
         <ns0:v>1027</ns0:v>
       </ns0:c>
       <ns0:c r="B516" t="s" s="0">
-        <ns0:v>4225</ns0:v>
+        <ns0:v>4774</ns0:v>
       </ns0:c>
       <ns0:c r="C516">
         <ns0:v>1</ns0:v>
@@ -38883,7 +41078,7 @@
         <ns0:v>1029</ns0:v>
       </ns0:c>
       <ns0:c r="B517" t="s" s="0">
-        <ns0:v>4226</ns0:v>
+        <ns0:v>4775</ns0:v>
       </ns0:c>
       <ns0:c r="C517">
         <ns0:v>0</ns0:v>
@@ -38900,7 +41095,7 @@
         <ns0:v>1031</ns0:v>
       </ns0:c>
       <ns0:c r="B518" t="s" s="0">
-        <ns0:v>4227</ns0:v>
+        <ns0:v>4776</ns0:v>
       </ns0:c>
       <ns0:c r="C518">
         <ns0:v>0</ns0:v>
@@ -38917,7 +41112,7 @@
         <ns0:v>1033</ns0:v>
       </ns0:c>
       <ns0:c r="B519" t="s" s="0">
-        <ns0:v>4228</ns0:v>
+        <ns0:v>4777</ns0:v>
       </ns0:c>
       <ns0:c r="C519">
         <ns0:v>11</ns0:v>
@@ -38934,7 +41129,7 @@
         <ns0:v>1034</ns0:v>
       </ns0:c>
       <ns0:c r="B520" t="s" s="0">
-        <ns0:v>4229</ns0:v>
+        <ns0:v>4778</ns0:v>
       </ns0:c>
       <ns0:c r="C520">
         <ns0:v>0</ns0:v>
@@ -39002,7 +41197,7 @@
         <ns0:v>1042</ns0:v>
       </ns0:c>
       <ns0:c r="B524" t="s" s="0">
-        <ns0:v>4230</ns0:v>
+        <ns0:v>4779</ns0:v>
       </ns0:c>
       <ns0:c r="C524">
         <ns0:v>0</ns0:v>
@@ -39019,7 +41214,7 @@
         <ns0:v>1044</ns0:v>
       </ns0:c>
       <ns0:c r="B525" t="s" s="0">
-        <ns0:v>4231</ns0:v>
+        <ns0:v>4780</ns0:v>
       </ns0:c>
       <ns0:c r="C525">
         <ns0:v>0</ns0:v>
@@ -39070,7 +41265,7 @@
         <ns0:v>1050</ns0:v>
       </ns0:c>
       <ns0:c r="B528" t="s" s="0">
-        <ns0:v>4232</ns0:v>
+        <ns0:v>4781</ns0:v>
       </ns0:c>
       <ns0:c r="C528">
         <ns0:v>0</ns0:v>
@@ -39138,7 +41333,7 @@
         <ns0:v>1058</ns0:v>
       </ns0:c>
       <ns0:c r="B532" t="s" s="0">
-        <ns0:v>4233</ns0:v>
+        <ns0:v>4782</ns0:v>
       </ns0:c>
       <ns0:c r="C532">
         <ns0:v>2</ns0:v>
@@ -39257,7 +41452,7 @@
         <ns0:v>1072</ns0:v>
       </ns0:c>
       <ns0:c r="B539" t="s" s="0">
-        <ns0:v>4234</ns0:v>
+        <ns0:v>4783</ns0:v>
       </ns0:c>
       <ns0:c r="C539">
         <ns0:v>3</ns0:v>
@@ -39308,7 +41503,7 @@
         <ns0:v>1078</ns0:v>
       </ns0:c>
       <ns0:c r="B542" t="s" s="0">
-        <ns0:v>4235</ns0:v>
+        <ns0:v>4784</ns0:v>
       </ns0:c>
       <ns0:c r="C542">
         <ns0:v>0</ns0:v>
@@ -39444,7 +41639,7 @@
         <ns0:v>1093</ns0:v>
       </ns0:c>
       <ns0:c r="B550" t="s" s="0">
-        <ns0:v>4237</ns0:v>
+        <ns0:v>4785</ns0:v>
       </ns0:c>
       <ns0:c r="C550">
         <ns0:v>3</ns0:v>
@@ -39461,7 +41656,7 @@
         <ns0:v>1095</ns0:v>
       </ns0:c>
       <ns0:c r="B551" t="s" s="0">
-        <ns0:v>4238</ns0:v>
+        <ns0:v>4786</ns0:v>
       </ns0:c>
       <ns0:c r="C551">
         <ns0:v>2</ns0:v>
@@ -39478,7 +41673,7 @@
         <ns0:v>1097</ns0:v>
       </ns0:c>
       <ns0:c r="B552" t="s" s="0">
-        <ns0:v>4239</ns0:v>
+        <ns0:v>4787</ns0:v>
       </ns0:c>
       <ns0:c r="C552">
         <ns0:v>1</ns0:v>
@@ -39495,7 +41690,7 @@
         <ns0:v>1099</ns0:v>
       </ns0:c>
       <ns0:c r="B553" t="s" s="0">
-        <ns0:v>4240</ns0:v>
+        <ns0:v>4788</ns0:v>
       </ns0:c>
       <ns0:c r="C553">
         <ns0:v>162</ns0:v>
@@ -39563,7 +41758,7 @@
         <ns0:v>1107</ns0:v>
       </ns0:c>
       <ns0:c r="B557" t="s" s="0">
-        <ns0:v>4241</ns0:v>
+        <ns0:v>4789</ns0:v>
       </ns0:c>
       <ns0:c r="C557">
         <ns0:v>3</ns0:v>
@@ -39580,7 +41775,7 @@
         <ns0:v>1109</ns0:v>
       </ns0:c>
       <ns0:c r="B558" t="s" s="0">
-        <ns0:v>4242</ns0:v>
+        <ns0:v>4790</ns0:v>
       </ns0:c>
       <ns0:c r="C558">
         <ns0:v>36</ns0:v>
@@ -39648,7 +41843,7 @@
         <ns0:v>1115</ns0:v>
       </ns0:c>
       <ns0:c r="B562" t="s" s="0">
-        <ns0:v>4244</ns0:v>
+        <ns0:v>4791</ns0:v>
       </ns0:c>
       <ns0:c r="C562">
         <ns0:v>1</ns0:v>
@@ -39733,7 +41928,7 @@
         <ns0:v>1125</ns0:v>
       </ns0:c>
       <ns0:c r="B567" t="s" s="0">
-        <ns0:v>4245</ns0:v>
+        <ns0:v>4792</ns0:v>
       </ns0:c>
       <ns0:c r="C567">
         <ns0:v>2</ns0:v>
@@ -39750,7 +41945,7 @@
         <ns0:v>1127</ns0:v>
       </ns0:c>
       <ns0:c r="B568" t="s" s="0">
-        <ns0:v>4246</ns0:v>
+        <ns0:v>4793</ns0:v>
       </ns0:c>
       <ns0:c r="C568">
         <ns0:v>1</ns0:v>
@@ -39818,7 +42013,7 @@
         <ns0:v>1135</ns0:v>
       </ns0:c>
       <ns0:c r="B572" t="s" s="0">
-        <ns0:v>4247</ns0:v>
+        <ns0:v>4794</ns0:v>
       </ns0:c>
       <ns0:c r="C572">
         <ns0:v>0</ns0:v>
@@ -39869,7 +42064,7 @@
         <ns0:v>1141</ns0:v>
       </ns0:c>
       <ns0:c r="B575" t="s" s="0">
-        <ns0:v>4248</ns0:v>
+        <ns0:v>4795</ns0:v>
       </ns0:c>
       <ns0:c r="C575">
         <ns0:v>3</ns0:v>
@@ -39886,7 +42081,7 @@
         <ns0:v>1143</ns0:v>
       </ns0:c>
       <ns0:c r="B576" t="s" s="0">
-        <ns0:v>4249</ns0:v>
+        <ns0:v>4796</ns0:v>
       </ns0:c>
       <ns0:c r="C576">
         <ns0:v>2</ns0:v>
@@ -39903,7 +42098,7 @@
         <ns0:v>1144</ns0:v>
       </ns0:c>
       <ns0:c r="B577" t="s" s="0">
-        <ns0:v>4250</ns0:v>
+        <ns0:v>4797</ns0:v>
       </ns0:c>
       <ns0:c r="C577">
         <ns0:v>1</ns0:v>
@@ -39920,7 +42115,7 @@
         <ns0:v>1145</ns0:v>
       </ns0:c>
       <ns0:c r="B578" t="s" s="0">
-        <ns0:v>4251</ns0:v>
+        <ns0:v>4798</ns0:v>
       </ns0:c>
       <ns0:c r="C578">
         <ns0:v>1</ns0:v>
@@ -39937,7 +42132,7 @@
         <ns0:v>1147</ns0:v>
       </ns0:c>
       <ns0:c r="B579" t="s" s="0">
-        <ns0:v>4252</ns0:v>
+        <ns0:v>4799</ns0:v>
       </ns0:c>
       <ns0:c r="C579">
         <ns0:v>2</ns0:v>
@@ -39954,7 +42149,7 @@
         <ns0:v>1149</ns0:v>
       </ns0:c>
       <ns0:c r="B580" t="s" s="0">
-        <ns0:v>4253</ns0:v>
+        <ns0:v>4800</ns0:v>
       </ns0:c>
       <ns0:c r="C580">
         <ns0:v>1</ns0:v>
@@ -39971,7 +42166,7 @@
         <ns0:v>1151</ns0:v>
       </ns0:c>
       <ns0:c r="B581" t="s" s="0">
-        <ns0:v>4254</ns0:v>
+        <ns0:v>4801</ns0:v>
       </ns0:c>
       <ns0:c r="C581">
         <ns0:v>6</ns0:v>
@@ -40090,7 +42285,7 @@
         <ns0:v>1165</ns0:v>
       </ns0:c>
       <ns0:c r="B588" t="s" s="0">
-        <ns0:v>4255</ns0:v>
+        <ns0:v>4802</ns0:v>
       </ns0:c>
       <ns0:c r="C588">
         <ns0:v>0</ns0:v>
@@ -40192,7 +42387,7 @@
         <ns0:v>1177</ns0:v>
       </ns0:c>
       <ns0:c r="B594" t="s" s="0">
-        <ns0:v>4256</ns0:v>
+        <ns0:v>4803</ns0:v>
       </ns0:c>
       <ns0:c r="C594">
         <ns0:v>0</ns0:v>
@@ -40294,7 +42489,7 @@
         <ns0:v>1189</ns0:v>
       </ns0:c>
       <ns0:c r="B600" t="s" s="0">
-        <ns0:v>4257</ns0:v>
+        <ns0:v>4804</ns0:v>
       </ns0:c>
       <ns0:c r="C600">
         <ns0:v>2</ns0:v>
@@ -40311,7 +42506,7 @@
         <ns0:v>1191</ns0:v>
       </ns0:c>
       <ns0:c r="B601" t="s" s="0">
-        <ns0:v>4258</ns0:v>
+        <ns0:v>4805</ns0:v>
       </ns0:c>
       <ns0:c r="C601">
         <ns0:v>0</ns0:v>
@@ -40345,7 +42540,7 @@
         <ns0:v>1195</ns0:v>
       </ns0:c>
       <ns0:c r="B603" t="s" s="0">
-        <ns0:v>4259</ns0:v>
+        <ns0:v>4806</ns0:v>
       </ns0:c>
       <ns0:c r="C603">
         <ns0:v>6</ns0:v>
@@ -40379,7 +42574,7 @@
         <ns0:v>1199</ns0:v>
       </ns0:c>
       <ns0:c r="B605" t="s" s="0">
-        <ns0:v>4260</ns0:v>
+        <ns0:v>4807</ns0:v>
       </ns0:c>
       <ns0:c r="C605">
         <ns0:v>2</ns0:v>
@@ -40430,7 +42625,7 @@
         <ns0:v>1205</ns0:v>
       </ns0:c>
       <ns0:c r="B608" t="s" s="0">
-        <ns0:v>4261</ns0:v>
+        <ns0:v>4808</ns0:v>
       </ns0:c>
       <ns0:c r="C608">
         <ns0:v>0</ns0:v>
@@ -40447,7 +42642,7 @@
         <ns0:v>1207</ns0:v>
       </ns0:c>
       <ns0:c r="B609" t="s" s="0">
-        <ns0:v>4262</ns0:v>
+        <ns0:v>4809</ns0:v>
       </ns0:c>
       <ns0:c r="C609">
         <ns0:v>2</ns0:v>
@@ -40464,7 +42659,7 @@
         <ns0:v>1209</ns0:v>
       </ns0:c>
       <ns0:c r="B610" t="s" s="0">
-        <ns0:v>4263</ns0:v>
+        <ns0:v>4810</ns0:v>
       </ns0:c>
       <ns0:c r="C610">
         <ns0:v>0</ns0:v>
@@ -40498,7 +42693,7 @@
         <ns0:v>1213</ns0:v>
       </ns0:c>
       <ns0:c r="B612" t="s" s="0">
-        <ns0:v>4264</ns0:v>
+        <ns0:v>4811</ns0:v>
       </ns0:c>
       <ns0:c r="C612">
         <ns0:v>0</ns0:v>
@@ -40515,7 +42710,7 @@
         <ns0:v>1214</ns0:v>
       </ns0:c>
       <ns0:c r="B613" t="s" s="0">
-        <ns0:v>4265</ns0:v>
+        <ns0:v>4812</ns0:v>
       </ns0:c>
       <ns0:c r="C613">
         <ns0:v>2</ns0:v>
@@ -40532,7 +42727,7 @@
         <ns0:v>1216</ns0:v>
       </ns0:c>
       <ns0:c r="B614" t="s" s="0">
-        <ns0:v>4266</ns0:v>
+        <ns0:v>4813</ns0:v>
       </ns0:c>
       <ns0:c r="C614">
         <ns0:v>0</ns0:v>
@@ -40549,7 +42744,7 @@
         <ns0:v>1218</ns0:v>
       </ns0:c>
       <ns0:c r="B615" t="s" s="0">
-        <ns0:v>4267</ns0:v>
+        <ns0:v>4814</ns0:v>
       </ns0:c>
       <ns0:c r="C615">
         <ns0:v>0</ns0:v>
@@ -40566,7 +42761,7 @@
         <ns0:v>1220</ns0:v>
       </ns0:c>
       <ns0:c r="B616" t="s" s="0">
-        <ns0:v>4268</ns0:v>
+        <ns0:v>4815</ns0:v>
       </ns0:c>
       <ns0:c r="C616">
         <ns0:v>1</ns0:v>
@@ -40583,7 +42778,7 @@
         <ns0:v>1222</ns0:v>
       </ns0:c>
       <ns0:c r="B617" t="s" s="0">
-        <ns0:v>4269</ns0:v>
+        <ns0:v>4816</ns0:v>
       </ns0:c>
       <ns0:c r="C617">
         <ns0:v>1</ns0:v>
@@ -40634,7 +42829,7 @@
         <ns0:v>1228</ns0:v>
       </ns0:c>
       <ns0:c r="B620" t="s" s="0">
-        <ns0:v>4270</ns0:v>
+        <ns0:v>4817</ns0:v>
       </ns0:c>
       <ns0:c r="C620">
         <ns0:v>1</ns0:v>
@@ -40702,7 +42897,7 @@
         <ns0:v>1235</ns0:v>
       </ns0:c>
       <ns0:c r="B624" t="s" s="0">
-        <ns0:v>4271</ns0:v>
+        <ns0:v>4818</ns0:v>
       </ns0:c>
       <ns0:c r="C624">
         <ns0:v>1</ns0:v>
@@ -40736,7 +42931,7 @@
         <ns0:v>1239</ns0:v>
       </ns0:c>
       <ns0:c r="B626" t="s" s="0">
-        <ns0:v>4272</ns0:v>
+        <ns0:v>4819</ns0:v>
       </ns0:c>
       <ns0:c r="C626">
         <ns0:v>1</ns0:v>
@@ -40753,7 +42948,7 @@
         <ns0:v>1241</ns0:v>
       </ns0:c>
       <ns0:c r="B627" t="s" s="0">
-        <ns0:v>4273</ns0:v>
+        <ns0:v>4820</ns0:v>
       </ns0:c>
       <ns0:c r="C627">
         <ns0:v>0</ns0:v>
@@ -40770,7 +42965,7 @@
         <ns0:v>1243</ns0:v>
       </ns0:c>
       <ns0:c r="B628" t="s" s="0">
-        <ns0:v>4274</ns0:v>
+        <ns0:v>4821</ns0:v>
       </ns0:c>
       <ns0:c r="C628">
         <ns0:v>0</ns0:v>
@@ -40838,7 +43033,7 @@
         <ns0:v>1250</ns0:v>
       </ns0:c>
       <ns0:c r="B632" t="s" s="0">
-        <ns0:v>4275</ns0:v>
+        <ns0:v>4822</ns0:v>
       </ns0:c>
       <ns0:c r="C632">
         <ns0:v>2</ns0:v>
@@ -40872,7 +43067,7 @@
         <ns0:v>1254</ns0:v>
       </ns0:c>
       <ns0:c r="B634" t="s" s="0">
-        <ns0:v>4276</ns0:v>
+        <ns0:v>4823</ns0:v>
       </ns0:c>
       <ns0:c r="C634">
         <ns0:v>3</ns0:v>
@@ -40889,7 +43084,7 @@
         <ns0:v>1256</ns0:v>
       </ns0:c>
       <ns0:c r="B635" t="s" s="0">
-        <ns0:v>4277</ns0:v>
+        <ns0:v>4824</ns0:v>
       </ns0:c>
       <ns0:c r="C635">
         <ns0:v>0</ns0:v>
@@ -40906,7 +43101,7 @@
         <ns0:v>1258</ns0:v>
       </ns0:c>
       <ns0:c r="B636" t="s" s="0">
-        <ns0:v>4278</ns0:v>
+        <ns0:v>4825</ns0:v>
       </ns0:c>
       <ns0:c r="C636">
         <ns0:v>1</ns0:v>
@@ -40923,7 +43118,7 @@
         <ns0:v>1260</ns0:v>
       </ns0:c>
       <ns0:c r="B637" t="s" s="0">
-        <ns0:v>4279</ns0:v>
+        <ns0:v>4826</ns0:v>
       </ns0:c>
       <ns0:c r="C637">
         <ns0:v>0</ns0:v>
@@ -40940,7 +43135,7 @@
         <ns0:v>1262</ns0:v>
       </ns0:c>
       <ns0:c r="B638" t="s" s="0">
-        <ns0:v>4280</ns0:v>
+        <ns0:v>4827</ns0:v>
       </ns0:c>
       <ns0:c r="C638">
         <ns0:v>0</ns0:v>
@@ -40974,7 +43169,7 @@
         <ns0:v>1266</ns0:v>
       </ns0:c>
       <ns0:c r="B640" t="s" s="0">
-        <ns0:v>4281</ns0:v>
+        <ns0:v>4828</ns0:v>
       </ns0:c>
       <ns0:c r="C640">
         <ns0:v>3</ns0:v>
@@ -40991,7 +43186,7 @@
         <ns0:v>1268</ns0:v>
       </ns0:c>
       <ns0:c r="B641" t="s" s="0">
-        <ns0:v>4282</ns0:v>
+        <ns0:v>4829</ns0:v>
       </ns0:c>
       <ns0:c r="C641">
         <ns0:v>0</ns0:v>
@@ -41178,7 +43373,7 @@
         <ns0:v>1288</ns0:v>
       </ns0:c>
       <ns0:c r="B652" t="s" s="0">
-        <ns0:v>4283</ns0:v>
+        <ns0:v>4830</ns0:v>
       </ns0:c>
       <ns0:c r="C652">
         <ns0:v>0</ns0:v>
@@ -41212,7 +43407,7 @@
         <ns0:v>1292</ns0:v>
       </ns0:c>
       <ns0:c r="B654" t="s" s="0">
-        <ns0:v>4284</ns0:v>
+        <ns0:v>4831</ns0:v>
       </ns0:c>
       <ns0:c r="C654">
         <ns0:v>5</ns0:v>
@@ -41229,7 +43424,7 @@
         <ns0:v>1294</ns0:v>
       </ns0:c>
       <ns0:c r="B655" t="s" s="0">
-        <ns0:v>4285</ns0:v>
+        <ns0:v>4832</ns0:v>
       </ns0:c>
       <ns0:c r="C655">
         <ns0:v>4</ns0:v>
@@ -41263,7 +43458,7 @@
         <ns0:v>1298</ns0:v>
       </ns0:c>
       <ns0:c r="B657" t="s" s="0">
-        <ns0:v>4286</ns0:v>
+        <ns0:v>4833</ns0:v>
       </ns0:c>
       <ns0:c r="C657">
         <ns0:v>3</ns0:v>
@@ -41314,7 +43509,7 @@
         <ns0:v>1303</ns0:v>
       </ns0:c>
       <ns0:c r="B660" t="s" s="0">
-        <ns0:v>4287</ns0:v>
+        <ns0:v>4834</ns0:v>
       </ns0:c>
       <ns0:c r="C660">
         <ns0:v>2</ns0:v>
@@ -41331,7 +43526,7 @@
         <ns0:v>1305</ns0:v>
       </ns0:c>
       <ns0:c r="B661" t="s" s="0">
-        <ns0:v>4288</ns0:v>
+        <ns0:v>4835</ns0:v>
       </ns0:c>
       <ns0:c r="C661">
         <ns0:v>7</ns0:v>
@@ -41399,7 +43594,7 @@
         <ns0:v>1311</ns0:v>
       </ns0:c>
       <ns0:c r="B665" t="s" s="0">
-        <ns0:v>4289</ns0:v>
+        <ns0:v>4836</ns0:v>
       </ns0:c>
       <ns0:c r="C665">
         <ns0:v>0</ns0:v>
@@ -41433,7 +43628,7 @@
         <ns0:v>1316</ns0:v>
       </ns0:c>
       <ns0:c r="B667" t="s" s="0">
-        <ns0:v>4290</ns0:v>
+        <ns0:v>4837</ns0:v>
       </ns0:c>
       <ns0:c r="C667">
         <ns0:v>2</ns0:v>
@@ -41501,7 +43696,7 @@
         <ns0:v>1324</ns0:v>
       </ns0:c>
       <ns0:c r="B671" t="s" s="0">
-        <ns0:v>4291</ns0:v>
+        <ns0:v>4838</ns0:v>
       </ns0:c>
       <ns0:c r="C671">
         <ns0:v>0</ns0:v>
@@ -41518,7 +43713,7 @@
         <ns0:v>1326</ns0:v>
       </ns0:c>
       <ns0:c r="B672" t="s" s="0">
-        <ns0:v>4292</ns0:v>
+        <ns0:v>4839</ns0:v>
       </ns0:c>
       <ns0:c r="C672">
         <ns0:v>0</ns0:v>
@@ -41535,7 +43730,7 @@
         <ns0:v>1328</ns0:v>
       </ns0:c>
       <ns0:c r="B673" t="s" s="0">
-        <ns0:v>4293</ns0:v>
+        <ns0:v>4840</ns0:v>
       </ns0:c>
       <ns0:c r="C673">
         <ns0:v>1</ns0:v>
@@ -41586,7 +43781,7 @@
         <ns0:v>1334</ns0:v>
       </ns0:c>
       <ns0:c r="B676" t="s" s="0">
-        <ns0:v>4294</ns0:v>
+        <ns0:v>4841</ns0:v>
       </ns0:c>
       <ns0:c r="C676">
         <ns0:v>0</ns0:v>
@@ -41603,7 +43798,7 @@
         <ns0:v>1336</ns0:v>
       </ns0:c>
       <ns0:c r="B677" t="s" s="0">
-        <ns0:v>4295</ns0:v>
+        <ns0:v>4842</ns0:v>
       </ns0:c>
       <ns0:c r="C677">
         <ns0:v>1</ns0:v>
@@ -41620,7 +43815,7 @@
         <ns0:v>1338</ns0:v>
       </ns0:c>
       <ns0:c r="B678" t="s" s="0">
-        <ns0:v>4296</ns0:v>
+        <ns0:v>4843</ns0:v>
       </ns0:c>
       <ns0:c r="C678">
         <ns0:v>2</ns0:v>
@@ -41671,7 +43866,7 @@
         <ns0:v>1344</ns0:v>
       </ns0:c>
       <ns0:c r="B681" t="s" s="0">
-        <ns0:v>4297</ns0:v>
+        <ns0:v>4844</ns0:v>
       </ns0:c>
       <ns0:c r="C681">
         <ns0:v>7</ns0:v>
@@ -41705,7 +43900,7 @@
         <ns0:v>1348</ns0:v>
       </ns0:c>
       <ns0:c r="B683" t="s" s="0">
-        <ns0:v>4298</ns0:v>
+        <ns0:v>4845</ns0:v>
       </ns0:c>
       <ns0:c r="C683">
         <ns0:v>0</ns0:v>
@@ -41892,7 +44087,7 @@
         <ns0:v>1369</ns0:v>
       </ns0:c>
       <ns0:c r="B694" t="s" s="0">
-        <ns0:v>4299</ns0:v>
+        <ns0:v>4676</ns0:v>
       </ns0:c>
       <ns0:c r="C694">
         <ns0:v>1</ns0:v>
@@ -41926,7 +44121,7 @@
         <ns0:v>1372</ns0:v>
       </ns0:c>
       <ns0:c r="B696" t="s" s="0">
-        <ns0:v>4300</ns0:v>
+        <ns0:v>4846</ns0:v>
       </ns0:c>
       <ns0:c r="C696">
         <ns0:v>2</ns0:v>
@@ -41943,7 +44138,7 @@
         <ns0:v>1374</ns0:v>
       </ns0:c>
       <ns0:c r="B697" t="s" s="0">
-        <ns0:v>4301</ns0:v>
+        <ns0:v>4847</ns0:v>
       </ns0:c>
       <ns0:c r="C697">
         <ns0:v>1</ns0:v>
@@ -41994,7 +44189,7 @@
         <ns0:v>1380</ns0:v>
       </ns0:c>
       <ns0:c r="B700" t="s" s="0">
-        <ns0:v>4302</ns0:v>
+        <ns0:v>4848</ns0:v>
       </ns0:c>
       <ns0:c r="C700">
         <ns0:v>2</ns0:v>
@@ -42062,7 +44257,7 @@
         <ns0:v>1387</ns0:v>
       </ns0:c>
       <ns0:c r="B704" t="s" s="0">
-        <ns0:v>4303</ns0:v>
+        <ns0:v>4849</ns0:v>
       </ns0:c>
       <ns0:c r="C704">
         <ns0:v>0</ns0:v>
@@ -42079,7 +44274,7 @@
         <ns0:v>1388</ns0:v>
       </ns0:c>
       <ns0:c r="B705" t="s" s="0">
-        <ns0:v>4304</ns0:v>
+        <ns0:v>4850</ns0:v>
       </ns0:c>
       <ns0:c r="C705">
         <ns0:v>1</ns0:v>
@@ -42419,7 +44614,7 @@
         <ns0:v>1428</ns0:v>
       </ns0:c>
       <ns0:c r="B725" t="s" s="0">
-        <ns0:v>4305</ns0:v>
+        <ns0:v>4851</ns0:v>
       </ns0:c>
       <ns0:c r="C725">
         <ns0:v>4</ns0:v>
@@ -42572,7 +44767,7 @@
         <ns0:v>1446</ns0:v>
       </ns0:c>
       <ns0:c r="B734" t="s" s="0">
-        <ns0:v>4306</ns0:v>
+        <ns0:v>4852</ns0:v>
       </ns0:c>
       <ns0:c r="C734">
         <ns0:v>2</ns0:v>
@@ -42742,7 +44937,7 @@
         <ns0:v>1465</ns0:v>
       </ns0:c>
       <ns0:c r="B744" t="s" s="0">
-        <ns0:v>4307</ns0:v>
+        <ns0:v>4853</ns0:v>
       </ns0:c>
       <ns0:c r="C744">
         <ns0:v>1</ns0:v>
@@ -42759,7 +44954,7 @@
         <ns0:v>1467</ns0:v>
       </ns0:c>
       <ns0:c r="B745" t="s" s="0">
-        <ns0:v>4308</ns0:v>
+        <ns0:v>4854</ns0:v>
       </ns0:c>
       <ns0:c r="C745">
         <ns0:v>1</ns0:v>
@@ -42776,7 +44971,7 @@
         <ns0:v>1468</ns0:v>
       </ns0:c>
       <ns0:c r="B746" t="s" s="0">
-        <ns0:v>4309</ns0:v>
+        <ns0:v>4855</ns0:v>
       </ns0:c>
       <ns0:c r="C746">
         <ns0:v>2</ns0:v>
@@ -42810,7 +45005,7 @@
         <ns0:v>1472</ns0:v>
       </ns0:c>
       <ns0:c r="B748" t="s" s="0">
-        <ns0:v>4310</ns0:v>
+        <ns0:v>4856</ns0:v>
       </ns0:c>
       <ns0:c r="C748">
         <ns0:v>1</ns0:v>
@@ -43014,7 +45209,7 @@
         <ns0:v>1495</ns0:v>
       </ns0:c>
       <ns0:c r="B760" t="s" s="0">
-        <ns0:v>4311</ns0:v>
+        <ns0:v>4857</ns0:v>
       </ns0:c>
       <ns0:c r="C760">
         <ns0:v>3</ns0:v>
@@ -43082,7 +45277,7 @@
         <ns0:v>1503</ns0:v>
       </ns0:c>
       <ns0:c r="B764" t="s" s="0">
-        <ns0:v>4312</ns0:v>
+        <ns0:v>4858</ns0:v>
       </ns0:c>
       <ns0:c r="C764">
         <ns0:v>3</ns0:v>
@@ -43167,7 +45362,7 @@
         <ns0:v>1513</ns0:v>
       </ns0:c>
       <ns0:c r="B769" t="s" s="0">
-        <ns0:v>4313</ns0:v>
+        <ns0:v>4859</ns0:v>
       </ns0:c>
       <ns0:c r="C769">
         <ns0:v>1</ns0:v>
@@ -43218,7 +45413,7 @@
         <ns0:v>1519</ns0:v>
       </ns0:c>
       <ns0:c r="B772" t="s" s="0">
-        <ns0:v>4314</ns0:v>
+        <ns0:v>4860</ns0:v>
       </ns0:c>
       <ns0:c r="C772">
         <ns0:v>4</ns0:v>
@@ -43235,7 +45430,7 @@
         <ns0:v>1521</ns0:v>
       </ns0:c>
       <ns0:c r="B773" t="s" s="0">
-        <ns0:v>4315</ns0:v>
+        <ns0:v>4861</ns0:v>
       </ns0:c>
       <ns0:c r="C773">
         <ns0:v>1</ns0:v>
@@ -43252,7 +45447,7 @@
         <ns0:v>1523</ns0:v>
       </ns0:c>
       <ns0:c r="B774" t="s" s="0">
-        <ns0:v>4316</ns0:v>
+        <ns0:v>4862</ns0:v>
       </ns0:c>
       <ns0:c r="C774">
         <ns0:v>4</ns0:v>
@@ -43337,7 +45532,7 @@
         <ns0:v>1533</ns0:v>
       </ns0:c>
       <ns0:c r="B779" t="s" s="0">
-        <ns0:v>4317</ns0:v>
+        <ns0:v>4863</ns0:v>
       </ns0:c>
       <ns0:c r="C779">
         <ns0:v>1</ns0:v>
@@ -43354,7 +45549,7 @@
         <ns0:v>1535</ns0:v>
       </ns0:c>
       <ns0:c r="B780" t="s" s="0">
-        <ns0:v>4318</ns0:v>
+        <ns0:v>4864</ns0:v>
       </ns0:c>
       <ns0:c r="C780">
         <ns0:v>2</ns0:v>
@@ -43490,7 +45685,7 @@
         <ns0:v>1550</ns0:v>
       </ns0:c>
       <ns0:c r="B788" t="s" s="0">
-        <ns0:v>4319</ns0:v>
+        <ns0:v>4865</ns0:v>
       </ns0:c>
       <ns0:c r="C788">
         <ns0:v>2</ns0:v>
@@ -43626,7 +45821,7 @@
         <ns0:v>1566</ns0:v>
       </ns0:c>
       <ns0:c r="B796" t="s" s="0">
-        <ns0:v>4320</ns0:v>
+        <ns0:v>4866</ns0:v>
       </ns0:c>
       <ns0:c r="C796">
         <ns0:v>1</ns0:v>
@@ -43643,7 +45838,7 @@
         <ns0:v>1568</ns0:v>
       </ns0:c>
       <ns0:c r="B797" t="s" s="0">
-        <ns0:v>4321</ns0:v>
+        <ns0:v>4867</ns0:v>
       </ns0:c>
       <ns0:c r="C797">
         <ns0:v>2</ns0:v>
@@ -43813,7 +46008,7 @@
         <ns0:v>1588</ns0:v>
       </ns0:c>
       <ns0:c r="B807" t="s" s="0">
-        <ns0:v>4322</ns0:v>
+        <ns0:v>4868</ns0:v>
       </ns0:c>
       <ns0:c r="C807">
         <ns0:v>0</ns0:v>
@@ -43966,7 +46161,7 @@
         <ns0:v>1606</ns0:v>
       </ns0:c>
       <ns0:c r="B816" t="s" s="0">
-        <ns0:v>4323</ns0:v>
+        <ns0:v>4869</ns0:v>
       </ns0:c>
       <ns0:c r="C816">
         <ns0:v>0</ns0:v>
@@ -44000,7 +46195,7 @@
         <ns0:v>1610</ns0:v>
       </ns0:c>
       <ns0:c r="B818" t="s" s="0">
-        <ns0:v>4324</ns0:v>
+        <ns0:v>4870</ns0:v>
       </ns0:c>
       <ns0:c r="C818">
         <ns0:v>1</ns0:v>
@@ -44068,7 +46263,7 @@
         <ns0:v>1618</ns0:v>
       </ns0:c>
       <ns0:c r="B822" t="s" s="0">
-        <ns0:v>4325</ns0:v>
+        <ns0:v>4871</ns0:v>
       </ns0:c>
       <ns0:c r="C822">
         <ns0:v>2</ns0:v>
@@ -44119,7 +46314,7 @@
         <ns0:v>1624</ns0:v>
       </ns0:c>
       <ns0:c r="B825" t="s" s="0">
-        <ns0:v>4326</ns0:v>
+        <ns0:v>4872</ns0:v>
       </ns0:c>
       <ns0:c r="C825">
         <ns0:v>3</ns0:v>
@@ -44153,7 +46348,7 @@
         <ns0:v>1627</ns0:v>
       </ns0:c>
       <ns0:c r="B827" t="s" s="0">
-        <ns0:v>4327</ns0:v>
+        <ns0:v>4873</ns0:v>
       </ns0:c>
       <ns0:c r="C827">
         <ns0:v>2</ns0:v>
@@ -44323,7 +46518,7 @@
         <ns0:v>1647</ns0:v>
       </ns0:c>
       <ns0:c r="B837" t="s" s="0">
-        <ns0:v>4328</ns0:v>
+        <ns0:v>4874</ns0:v>
       </ns0:c>
       <ns0:c r="C837">
         <ns0:v>0</ns0:v>
@@ -44459,7 +46654,7 @@
         <ns0:v>1663</ns0:v>
       </ns0:c>
       <ns0:c r="B845" t="s" s="0">
-        <ns0:v>4329</ns0:v>
+        <ns0:v>4875</ns0:v>
       </ns0:c>
       <ns0:c r="C845">
         <ns0:v>0</ns0:v>
@@ -44578,7 +46773,7 @@
         <ns0:v>1677</ns0:v>
       </ns0:c>
       <ns0:c r="B852" t="s" s="0">
-        <ns0:v>4330</ns0:v>
+        <ns0:v>4876</ns0:v>
       </ns0:c>
       <ns0:c r="C852">
         <ns0:v>0</ns0:v>
@@ -44833,7 +47028,7 @@
         <ns0:v>1706</ns0:v>
       </ns0:c>
       <ns0:c r="B867" t="s" s="0">
-        <ns0:v>4331</ns0:v>
+        <ns0:v>4877</ns0:v>
       </ns0:c>
       <ns0:c r="C867">
         <ns0:v>8</ns0:v>
@@ -44986,7 +47181,7 @@
         <ns0:v>1724</ns0:v>
       </ns0:c>
       <ns0:c r="B876" t="s" s="0">
-        <ns0:v>4332</ns0:v>
+        <ns0:v>4878</ns0:v>
       </ns0:c>
       <ns0:c r="C876">
         <ns0:v>2</ns0:v>
@@ -45547,7 +47742,7 @@
         <ns0:v>1789</ns0:v>
       </ns0:c>
       <ns0:c r="B909" t="s" s="0">
-        <ns0:v>4333</ns0:v>
+        <ns0:v>4879</ns0:v>
       </ns0:c>
       <ns0:c r="C909">
         <ns0:v>1</ns0:v>
@@ -45564,7 +47759,7 @@
         <ns0:v>1791</ns0:v>
       </ns0:c>
       <ns0:c r="B910" t="s" s="0">
-        <ns0:v>4334</ns0:v>
+        <ns0:v>4880</ns0:v>
       </ns0:c>
       <ns0:c r="C910">
         <ns0:v>0</ns0:v>
@@ -45581,7 +47776,7 @@
         <ns0:v>1793</ns0:v>
       </ns0:c>
       <ns0:c r="B911" t="s" s="0">
-        <ns0:v>4335</ns0:v>
+        <ns0:v>4881</ns0:v>
       </ns0:c>
       <ns0:c r="C911">
         <ns0:v>0</ns0:v>
@@ -45598,7 +47793,7 @@
         <ns0:v>1795</ns0:v>
       </ns0:c>
       <ns0:c r="B912" t="s" s="0">
-        <ns0:v>4336</ns0:v>
+        <ns0:v>4882</ns0:v>
       </ns0:c>
       <ns0:c r="C912">
         <ns0:v>0</ns0:v>
@@ -45632,7 +47827,7 @@
         <ns0:v>1799</ns0:v>
       </ns0:c>
       <ns0:c r="B914" t="s" s="0">
-        <ns0:v>4337</ns0:v>
+        <ns0:v>4883</ns0:v>
       </ns0:c>
       <ns0:c r="C914">
         <ns0:v>1</ns0:v>
@@ -45683,7 +47878,7 @@
         <ns0:v>1805</ns0:v>
       </ns0:c>
       <ns0:c r="B917" t="s" s="0">
-        <ns0:v>4338</ns0:v>
+        <ns0:v>4884</ns0:v>
       </ns0:c>
       <ns0:c r="C917">
         <ns0:v>1</ns0:v>
@@ -45751,7 +47946,7 @@
         <ns0:v>1813</ns0:v>
       </ns0:c>
       <ns0:c r="B921" t="s" s="0">
-        <ns0:v>4339</ns0:v>
+        <ns0:v>4885</ns0:v>
       </ns0:c>
       <ns0:c r="C921">
         <ns0:v>0</ns0:v>
@@ -45768,7 +47963,7 @@
         <ns0:v>1815</ns0:v>
       </ns0:c>
       <ns0:c r="B922" t="s" s="0">
-        <ns0:v>4340</ns0:v>
+        <ns0:v>4886</ns0:v>
       </ns0:c>
       <ns0:c r="C922">
         <ns0:v>3</ns0:v>
@@ -45853,7 +48048,7 @@
         <ns0:v>1825</ns0:v>
       </ns0:c>
       <ns0:c r="B927" t="s" s="0">
-        <ns0:v>4341</ns0:v>
+        <ns0:v>4887</ns0:v>
       </ns0:c>
       <ns0:c r="C927">
         <ns0:v>1</ns0:v>
@@ -45870,7 +48065,7 @@
         <ns0:v>1827</ns0:v>
       </ns0:c>
       <ns0:c r="B928" t="s" s="0">
-        <ns0:v>4342</ns0:v>
+        <ns0:v>4888</ns0:v>
       </ns0:c>
       <ns0:c r="C928">
         <ns0:v>1</ns0:v>
@@ -45955,7 +48150,7 @@
         <ns0:v>1837</ns0:v>
       </ns0:c>
       <ns0:c r="B933" t="s" s="0">
-        <ns0:v>4343</ns0:v>
+        <ns0:v>4889</ns0:v>
       </ns0:c>
       <ns0:c r="C933">
         <ns0:v>0</ns0:v>
@@ -46108,7 +48303,7 @@
         <ns0:v>1855</ns0:v>
       </ns0:c>
       <ns0:c r="B942" t="s" s="0">
-        <ns0:v>4344</ns0:v>
+        <ns0:v>4890</ns0:v>
       </ns0:c>
       <ns0:c r="C942">
         <ns0:v>0</ns0:v>
@@ -46125,7 +48320,7 @@
         <ns0:v>1857</ns0:v>
       </ns0:c>
       <ns0:c r="B943" t="s" s="0">
-        <ns0:v>4345</ns0:v>
+        <ns0:v>4891</ns0:v>
       </ns0:c>
       <ns0:c r="C943">
         <ns0:v>2</ns0:v>
@@ -46193,7 +48388,7 @@
         <ns0:v>1865</ns0:v>
       </ns0:c>
       <ns0:c r="B947" t="s" s="0">
-        <ns0:v>4346</ns0:v>
+        <ns0:v>4892</ns0:v>
       </ns0:c>
       <ns0:c r="C947">
         <ns0:v>0</ns0:v>
@@ -46210,7 +48405,7 @@
         <ns0:v>1867</ns0:v>
       </ns0:c>
       <ns0:c r="B948" t="s" s="0">
-        <ns0:v>4347</ns0:v>
+        <ns0:v>4893</ns0:v>
       </ns0:c>
       <ns0:c r="C948">
         <ns0:v>6</ns0:v>
@@ -46295,7 +48490,7 @@
         <ns0:v>1876</ns0:v>
       </ns0:c>
       <ns0:c r="B953" t="s" s="0">
-        <ns0:v>4348</ns0:v>
+        <ns0:v>4894</ns0:v>
       </ns0:c>
       <ns0:c r="C953">
         <ns0:v>2</ns0:v>
@@ -52228,7 +54423,7 @@
         <ns0:v>2569</ns0:v>
       </ns0:c>
       <ns0:c r="B1302" t="s" s="0">
-        <ns0:v>4669</ns0:v>
+        <ns0:v>4677</ns0:v>
       </ns0:c>
       <ns0:c r="C1302">
         <ns0:v>0</ns0:v>
@@ -52245,7 +54440,7 @@
         <ns0:v>2571</ns0:v>
       </ns0:c>
       <ns0:c r="B1303" t="s" s="0">
-        <ns0:v>4670</ns0:v>
+        <ns0:v>4678</ns0:v>
       </ns0:c>
       <ns0:c r="C1303">
         <ns0:v>158</ns0:v>

</xml_diff>

<commit_message>
update post state and fix truncated posts
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4895" uniqueCount="4895">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4905" uniqueCount="4905">
   <si>
     <t>日付</t>
   </si>
@@ -32254,6 +32254,204 @@
 あなた程度の筋肉量で体脂肪率を10%以下にする必要はありません。
 バルクアップをして高重量を持ちましょう。
 単純に体重が重い方が高重量が扱いやすいので。</t>
+  </si>
+  <si>
+    <t>自己満男磨き(笑)と呼ばれている習慣を擁護します。  
+【オナ禁】
+ →健康的な射精頻度の方には効果なし。 
+でもオナ猿には効果的。 
+・ED改善 
+・自己管理能力の向上 
+・ジヒドロテストステロンの抑制  
+個人的には2日以上やるとびんこち〇ち〇になるため、 セスクの前にやっておきたい。  
+【瞑想】 
+→前頭前野を鍛え、やるべきタスクと向き合う力を育てる。 時間が長ければ長いほど効果的。 
+ドーパミン中毒全般に良い効果をもたらす。  ただ、そもそもスマホ中毒者が工夫無しで習慣化できるかは疑問。
+  【コールドシャワー】 
+→朝に浴びるとカフェインのような覚醒効果がある。 
+また、 
+・ドーパミンが数時間分泌
+ ・エンドルフィン分泌→鬱軽減 
+・アイシング効果 がある。  
+デメリットは 
+・筋肥大の抑制 
+・心臓病のリスク  
+【ジャーナル】 
+→タスク整理、アイデア出し、不安の整理、目標確認など様々な使い方が可能。  
+一日の終わりにポジティブな出来事を書きだすことにより、幸福度が上がることが研究で分かっている。  
+また、ADHDなどで注意散漫な人がタスク整理や目標確認などに使用すると効果的。  
+ただ、ジャーナルを書いて現実が何か変わることはないため行動とセットで行う事はマスト。  
+何事も「意味あるorない」の二元論ではなく、 
+正しく評価して自分に落とし込むことが重要。</t>
+  </si>
+  <si>
+    <t>「筋トレの時間がない」は甘え。
+俺が一日10時間労働の中、90分の筋トレができる理由はこれ↓
+【やめるべき行動】
+・ポルノ
+・ゲーム
+・女を追う
+・食事に迷う
+・服装に迷う
+・LINEを続ける
+・目的なしSNS
+【マルチタスク】
+・授業or仕事中に副業
+・散歩中、考え事
+・移動中、音声学習
+時間は無駄な行動を減らせば、いくらでも作れる</t>
+  </si>
+  <si>
+    <t>「筋トレの時間がない」は甘え。
+俺が一日10時間労働の中、90分の筋トレができる理由はこれ↓
+【やめるべき行動】
+・ポルノ
+・ゲーム
+・女を追う
+・食事に迷う
+・服装に迷う
+・LINEを続ける
+・目的なしSNS
+【マルチタスク】
+・授業or仕事中に副業
+・散歩中、考え事
+・移動中、音声学習
+時間は無駄な行動を減らせば、いくらでも作れる</t>
+  </si>
+  <si>
+    <t>自己満男磨き(笑)と呼ばれている習慣を擁護します。  
+【オナ禁】
+ →健康的な射精頻度の方には効果なし。 
+でもオナ猿には効果的。 
+・ED改善 
+・自己管理能力の向上 
+・ジヒドロテストステロンの抑制  
+個人的には2日以上やるとびんこち〇ち〇になるため、 セスクの前にやっておきたい。  
+【瞑想】 
+→前頭前野を鍛え、やるべきタスクと向き合う力を育てる。 時間が長ければ長いほど効果的。 
+ドーパミン中毒全般に良い効果をもたらす。  ただ、そもそもスマホ中毒者が工夫無しで習慣化できるかは疑問。
+  【コールドシャワー】 
+→朝に浴びるとカフェインのような覚醒効果がある。 
+また、 
+・ドーパミンが数時間分泌
+ ・エンドルフィン分泌→鬱軽減 
+・アイシング効果 がある。  
+デメリットは 
+・筋肥大の抑制 
+・心臓病のリスク  
+【ジャーナル】 
+→タスク整理、アイデア出し、不安の整理、目標確認など様々な使い方が可能。  
+一日の終わりにポジティブな出来事を書きだすことにより、幸福度が上がることが研究で分かっている。  
+また、ADHDなどで注意散漫な人がタスク整理や目標確認などに使用すると効果的。  
+ただ、ジャーナルを書いて現実が何か変わることはないため行動とセットで行う事はマスト。  
+何事も「意味あるorない」の二元論ではなく、 
+正しく評価して自分に落とし込むことが重要。</t>
+  </si>
+  <si>
+    <t>自己満男磨き(笑)と呼ばれている習慣を擁護します。  
+【オナ禁】
+ →健康的な射精頻度の方には効果なし。 
+でもオナ猿には効果的。 
+・ED改善 
+・自己管理能力の向上 
+・ジヒドロテストステロンの抑制  
+個人的には2日以上やるとびんこち〇ち〇になるため、 セスクの前にやっておきたい。  
+【瞑想】 
+→前頭前野を鍛え、やるべきタスクと向き合う力を育てる。 時間が長ければ長いほど効果的。 
+ドーパミン中毒全般に良い効果をもたらす。  ただ、そもそもスマホ中毒者が工夫無しで習慣化できるかは疑問。
+  【コールドシャワー】 
+→朝に浴びるとカフェインのような覚醒効果がある。 
+また、 
+・ドーパミンが数時間分泌
+ ・エンドルフィン分泌→鬱軽減 
+・アイシング効果 がある。  
+デメリットは 
+・筋肥大の抑制 
+・心臓病のリスク  
+【ジャーナル】 
+→タスク整理、アイデア出し、不安の整理、目標確認など様々な使い方が可能。  
+一日の終わりにポジティブな出来事を書きだすことにより、幸福度が上がることが研究で分かっている。  
+また、ADHDなどで注意散漫な人がタスク整理や目標確認などに使用すると効果的。  
+ただ、ジャーナルを書いて現実が何か変わることはないため行動とセットで行う事はマスト。  
+何事も「意味あるorない」の二元論ではなく、 
+正しく評価して自分に落とし込むことが重要。</t>
+  </si>
+  <si>
+    <t>「筋トレの時間がない」は甘え。
+俺が一日10時間労働の中、90分の筋トレができる理由はこれ↓
+【やめるべき行動】
+・ポルノ
+・ゲーム
+・女を追う
+・食事に迷う
+・服装に迷う
+・LINEを続ける
+・目的なしSNS
+【マルチタスク】
+・授業or仕事中に副業
+・散歩中、考え事
+・移動中、音声学習
+時間は無駄な行動を減らせば、いくらでも作れる</t>
+  </si>
+  <si>
+    <t>自己満男磨き(笑)と呼ばれている習慣を擁護します。  
+【オナ禁】
+ →健康的な射精頻度の方には効果なし。 
+でもオナ猿には効果的。 
+・ED改善 
+・自己管理能力の向上 
+・ジヒドロテストステロンの抑制  
+個人的には2日以上やるとびんこち〇ち〇になるため、 セスクの前にやっておきたい。  
+【瞑想】 
+→前頭前野を鍛え、やるべきタスクと向き合う力を育てる。 時間が長ければ長いほど効果的。 
+ドーパミン中毒全般に良い効果をもたらす。  ただ、そもそもスマホ中毒者が工夫無しで習慣化できるかは疑問。
+  【コールドシャワー】 
+→朝に浴びるとカフェインのような覚醒効果がある。 
+また、 
+・ドーパミンが数時間分泌
+ ・エンドルフィン分泌→鬱軽減 
+・アイシング効果 がある。  
+デメリットは 
+・筋肥大の抑制 
+・心臓病のリスク  
+【ジャーナル】 
+→タスク整理、アイデア出し、不安の整理、目標確認など様々な使い方が可能。  
+一日の終わりにポジティブな出来事を書きだすことにより、幸福度が上がることが研究で分かっている。  
+また、ADHDなどで注意散漫な人がタスク整理や目標確認などに使用すると効果的。  
+ただ、ジャーナルを書いて現実が何か変わることはないため行動とセットで行う事はマスト。  
+何事も「意味あるorない」の二元論ではなく、 
+正しく評価して自分に落とし込むことが重要。</t>
+  </si>
+  <si>
+    <t>努力できる環境を作る方法
+・自己啓発動画を音声学習
+・目標をPC、スマホの壁紙にする
+・デスクに目標を張る
+・エロ垢を全てブロック
+・ロールモデルのみフォロー
+・夜に翌日のToDoリスト
+俺がヒョロガリだった頃はインスタで
+ボディビルダーをフォローしまくって毎日見ていた。
+目標は持つだけでなく刷り込め。</t>
+  </si>
+  <si>
+    <t>ニートの方はドーパミン中毒を極めてください。
+いかに快楽主義がゴミであるかが分かってきます。
+私はニート時代に
+・毎日10時間ゲーム
+・毎日5回シコる
+・週末は深夜に海外サッカー観る
+を昼夜逆転しながら2年間やってました。
+結果、分かったことはドーパミン中毒的な快楽主義は虚しいということ。
+この期間があったからこそ、自己成長に喜びを感じる今の自分がいます。</t>
+  </si>
+  <si>
+    <t>筋トレの意外なメリットは「自分に100％集中する時間」が得られること。
+現代人はこれが足りていない。
+SNSで他人の応援・批判、他人が作ったコンテンツを消費して一日が終わる。
+筋トレは違う。
+フォーム・先週との比較・レスト中すべて自分と向き合わなければいけない。
+モテるため以前に筋トレは最強のマインドフルネス。</t>
   </si>
 </sst>
 </file>
@@ -38307,7 +38505,7 @@
         <ns0:v>705</ns0:v>
       </ns0:c>
       <ns0:c r="B354" t="s" s="0">
-        <ns0:v>706</ns0:v>
+        <ns0:v>4895</ns0:v>
       </ns0:c>
       <ns0:c r="C354">
         <ns0:v>0</ns0:v>
@@ -38936,7 +39134,7 @@
         <ns0:v>779</ns0:v>
       </ns0:c>
       <ns0:c r="B391" t="s" s="0">
-        <ns0:v>4675</ns0:v>
+        <ns0:v>4896</ns0:v>
       </ns0:c>
       <ns0:c r="C391">
         <ns0:v>145</ns0:v>
@@ -44087,7 +44285,7 @@
         <ns0:v>1369</ns0:v>
       </ns0:c>
       <ns0:c r="B694" t="s" s="0">
-        <ns0:v>4676</ns0:v>
+        <ns0:v>4897</ns0:v>
       </ns0:c>
       <ns0:c r="C694">
         <ns0:v>1</ns0:v>
@@ -54423,7 +54621,7 @@
         <ns0:v>2569</ns0:v>
       </ns0:c>
       <ns0:c r="B1302" t="s" s="0">
-        <ns0:v>4677</ns0:v>
+        <ns0:v>4898</ns0:v>
       </ns0:c>
       <ns0:c r="C1302">
         <ns0:v>0</ns0:v>
@@ -54440,7 +54638,7 @@
         <ns0:v>2571</ns0:v>
       </ns0:c>
       <ns0:c r="B1303" t="s" s="0">
-        <ns0:v>4678</ns0:v>
+        <ns0:v>4899</ns0:v>
       </ns0:c>
       <ns0:c r="C1303">
         <ns0:v>158</ns0:v>
@@ -55035,7 +55233,7 @@
         <ns0:v>2641</ns0:v>
       </ns0:c>
       <ns0:c r="B1338" t="s" s="0">
-        <ns0:v>4514</ns0:v>
+        <ns0:v>4902</ns0:v>
       </ns0:c>
       <ns0:c r="C1338">
         <ns0:v>9</ns0:v>
@@ -55120,7 +55318,7 @@
         <ns0:v>2651</ns0:v>
       </ns0:c>
       <ns0:c r="B1343" t="s" s="0">
-        <ns0:v>4516</ns0:v>
+        <ns0:v>4903</ns0:v>
       </ns0:c>
       <ns0:c r="C1343">
         <ns0:v>7783</ns0:v>
@@ -55341,7 +55539,7 @@
         <ns0:v>2677</ns0:v>
       </ns0:c>
       <ns0:c r="B1356" t="s" s="0">
-        <ns0:v>4520</ns0:v>
+        <ns0:v>4900</ns0:v>
       </ns0:c>
       <ns0:c r="C1356">
         <ns0:v>27</ns0:v>
@@ -57823,7 +58021,7 @@
         <ns0:v>2959</ns0:v>
       </ns0:c>
       <ns0:c r="B1502" t="s" s="0">
-        <ns0:v>4575</ns0:v>
+        <ns0:v>4904</ns0:v>
       </ns0:c>
       <ns0:c r="C1502">
         <ns0:v>114</ns0:v>
@@ -68074,7 +68272,7 @@
         <ns0:v>4096</ns0:v>
       </ns0:c>
       <ns0:c r="B2105" t="s" s="0">
-        <ns0:v>4652</ns0:v>
+        <ns0:v>4901</ns0:v>
       </ns0:c>
       <ns0:c r="C2105">
         <ns0:v>10</ns0:v>

</xml_diff>

<commit_message>
Add local image support for new posts; add conbini_egg.jpg
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2174"/>
+  <dimension ref="A1:G2174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,11 @@
       <c r="F1" t="inlineStr">
         <is>
           <t>reply_url</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>image_path</t>
         </is>
       </c>
     </row>
@@ -63020,7 +63025,11 @@
           <t>normal</t>
         </is>
       </c>
-      <c r="F2174" t="inlineStr"/>
+      <c r="G2174" t="inlineStr">
+        <is>
+          <t>images/conbini_egg.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix truncated posts: スマホ中毒/チー牛 full text restore
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -41586,7 +41586,11 @@
 ・必要なものだけ残す
 ・アプリを最小化する
 ・環境を整える
-意志で我慢するより… https://t.co/gqeeWCjSjC</t>
+意志で我慢するより
+仕組みでコントロールした方が現実的。
+デトックス＝対症療法
+ミニマリズム＝根本的治療
+元スマホ廃人の私はこの考え方を持ってから大きく変わった。</t>
         </is>
       </c>
       <c r="C1425" t="n">
@@ -41687,7 +41691,21 @@
 でも、現実は
 ・週3回、自宅で5分トレ
 ・外見磨きは清潔感だけ
-・「筋トレすればモテる」を信じアプローチを怠る。</t>
+・「筋トレすればモテる」を信じアプローチを怠る。
+この努力量では永遠にイケメンとは並べない。
+なぜなら、イケメンも努力しているから。
+しかも、イケメンは「才能＋10代からの積み上げ」がある。
+同じ努力量なら
+差は縮まらないどころか固定される。
+俺が童貞大学生の時は
+講義後に連絡先交換しまくってたし
+同時進行でアプリも複数やっていた。
+当然、自己完結の男磨きも継続。
+ヒョロガリだったから
+夜にうなされながら大量にご飯を食べていた。
+努力のベクトルが正しくても、
+絶対的な量をクリアしないと意味がない。
+意外と言う人は少ないので、このポストで気づけたあなたは有利。</t>
         </is>
       </c>
       <c r="C1428" t="n">

</xml_diff>

<commit_message>
Fix truncated post: 恋愛テク (7/26 19:00)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -44880,7 +44880,11 @@
 ・「優しい人がいい」
 ・「チャラいのは無理」
 でも行動を見ると違う。
-だから見るべきは発言＜行動。… https://t.co/9dy4am2NyT</t>
+だから見るべきは発言＜行動。
+都会でいい女を連れてる男を見ろ。
+浮気しまくっている芸能人を見ろ。
+女の言葉には必ずバイアスがかかる。
+言葉を信じるな。行動を観察しろ。</t>
         </is>
       </c>
       <c r="C1530" t="n">

</xml_diff>

<commit_message>
Fix truncated post: ヒョロガリ最初の一週間 (7/26 21:00)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -44951,7 +44951,14 @@
 ・体脂肪率15%以下 → 増量（+300〜500kcal）
 ここまでは1日でやる。
 【環境構築】
-・食事内容を固定（高タンパク）</t>
+・食事内容を固定（高タンパク）
+・毎日同じ時間に体重測定
+・ジム or 自重トレ環境を用意
+【行動】
+・週3以上筋トレ
+・体重を毎日記録
+・摂取カロリーを守る
+最初の1週間で"ブレない型"を作れ。</t>
         </is>
       </c>
       <c r="C1532" t="n">

</xml_diff>

<commit_message>
Add skincare post (2026-07-27)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2194"/>
+  <dimension ref="A1:G2195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63719,6 +63719,41 @@
         </is>
       </c>
     </row>
+    <row r="2195">
+      <c r="A2195" t="inlineStr">
+        <is>
+          <t>2026-07-27 00:00:00</t>
+        </is>
+      </c>
+      <c r="B2195" t="inlineStr">
+        <is>
+          <t>肌を綺麗にしたい男へ。
+意外と重要じゃなかったもの
+・化粧水
+・洗顔フォーム
+・枕カバーを洗う
+重要だったもの
+・先天性
+・睡眠
+・食事
+・運動
+・紫外線対策
+・禁煙禁酒
+・ジュース禁止
+身体の内側からケアすれば、かなり変わる。</t>
+        </is>
+      </c>
+      <c r="E2195" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2195" t="inlineStr">
+        <is>
+          <t>https://x.com/puregrinding23/status/2058145954361123021</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add smartphone addiction post (2026-07-27)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2195"/>
+  <dimension ref="A1:G2196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63754,6 +63754,34 @@
         </is>
       </c>
     </row>
+    <row r="2196">
+      <c r="A2196" t="inlineStr">
+        <is>
+          <t>2026-07-27 00:00:00</t>
+        </is>
+      </c>
+      <c r="B2196" t="inlineStr">
+        <is>
+          <t>スマホ廃人時代の私
+・朝スマホで1時間浪費
+・YouTube見ながら作業
+・スクリーンタイム10時間
+・シコリながら深夜に寝落ち
+これで「モテたい」「金持ちになりたい」とか言ってた。
+今考えたら「出来るわけないだろ」と思う。</t>
+        </is>
+      </c>
+      <c r="E2196" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2196" t="inlineStr">
+        <is>
+          <t>https://x.com/puregrinding23/status/2058145954361123021</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add weak mindset post (2026-07-27)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2196"/>
+  <dimension ref="A1:G2197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63782,6 +63782,33 @@
         </is>
       </c>
     </row>
+    <row r="2197">
+      <c r="A2197" t="inlineStr">
+        <is>
+          <t>2026-07-27 00:00:00</t>
+        </is>
+      </c>
+      <c r="B2197" t="inlineStr">
+        <is>
+          <t>弱者はやらない理由を探し始める。
+非モテほど「モテても意味ない」と言い出す。
+貧乏な人ほど金持ちになるデメリットを語る。
+筋トレ強度が低い人ほどオーバーワークを気にする。
+成し遂げてから悩めばいい。
+手にしてない者が語る資格はない。</t>
+        </is>
+      </c>
+      <c r="E2197" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="F2197" t="inlineStr">
+        <is>
+          <t>https://x.com/puregrinding23/status/2058145954361123021</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update posts: extend ち〇ぽ post, fix ビンビン full text
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -45399,7 +45399,8 @@
 ・性欲を努力に昇華する 
 ・性欲を支配し、女を選ぶ側に立つ
 英雄は色を好む。
-弱男も色を好む。</t>
+弱男も色を好む。
+両者の違いは性欲を支配するか、性欲に支配されるかである。</t>
         </is>
       </c>
       <c r="C1546" t="n">
@@ -53226,7 +53227,10 @@
 ⑥ストレス管理 
 →コルチゾールを減らす 
 ⑦オナ禁2〜7日 
-→やり過ぎは注意… https://t.co/d7oDlkPe8Q</t>
+→やり過ぎは注意 
+⑧ポルノ断ち 
+→生の女体を見た時の興奮度が増す 
+ナチュラルバイアグラhttps://t.co/d7oDlkPe8Q</t>
         </is>
       </c>
       <c r="C1810" t="n">

</xml_diff>

<commit_message>
Add 3 lines to 非モテポテンシャル post (row 1568)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -46029,7 +46029,10 @@
 歯列矯正やケアで見た目を整える、
 できることを“思い込み”でやってないだけ。
 もちろん遺伝子的限界はある。
-そこは割り切れ。</t>
+そこは割り切れ。
+ただ、大半はそこにすら到達してない。
+俺もこの思い込みで何年も無駄にした。
+動いたやつから現実が変わる。</t>
         </is>
       </c>
       <c r="C1568" t="n">

</xml_diff>

<commit_message>
Add 2 lines to 女友達のいる非モテ post (row 1569)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -46063,7 +46063,9 @@
 原因はほぼこれ。
 ・下心の隠しすぎ
 ・外見の決定的減点
-・女の影が見えない</t>
+・女の影が見えない
+一度、「友達」のラベルを張られたらほぼ剥がれない。
+半年以上はその女の前から姿を消し、レベル上げに徹しよう。</t>
         </is>
       </c>
       <c r="C1569" t="n">

</xml_diff>

<commit_message>
Add manual post 2026-08-18: 筋トレしてもモテない人は
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2203"/>
+  <dimension ref="A1:G2204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63977,6 +63977,38 @@
         </is>
       </c>
     </row>
+    <row r="2204">
+      <c r="A2204" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2204" t="inlineStr">
+        <is>
+          <t>筋トレしてもモテない人は、
+・顔
+・身長
+・鎖骨の長さ
+・脚の長さ
+これらが極端に劣ってる。
+筋トレは間違いなくプラスになるけど、
+期待しすぎない方が良いね。
+俺自身、自閉症チー牛からモテ攻略できた。
+筋トレで体重39kgから倍近く増やしたけど、やってきたのはそれだけじゃない。</t>
+        </is>
+      </c>
+      <c r="C2204" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2204" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2204" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add manual post 2026-08-18: 真のスコットランド人論法
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2205"/>
+  <dimension ref="A1:G2206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64046,6 +64046,37 @@
         </is>
       </c>
     </row>
+    <row r="2206">
+      <c r="A2206" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2206" t="inlineStr">
+        <is>
+          <t>都合が悪くなったら、 
+「真の○○は..」と言って勝手に言葉の定義狭めてくる奴、マジで嫌い。  
+（真のスコットランド人論法）
+「真の陽キャは群れない」
+「真の強者は他人を見下さない」
+「本当のマッチョは優しい」
+これ系弱者根性過ぎる😅
+現実を見よう。
+認めたくないのは分かるけども。</t>
+        </is>
+      </c>
+      <c r="C2206" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2206" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2206" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-08-24 (童貞が美女攻略)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2214"/>
+  <dimension ref="A1:G2215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64358,6 +64358,37 @@
         </is>
       </c>
     </row>
+    <row r="2215">
+      <c r="A2215" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B2215" t="inlineStr">
+        <is>
+          <t>童貞が「美女攻略」を考えない方がいい。
+むしろブス、BBA、ニューハーフを片っ端から当たれ。
+誘い方
+拒絶
+距離の縮め方
+クロージング
+経験を積んでいないと、いざ本命が現れた時に何もできない。「好きな人にだけ好かれればいい」は机上の空論。
+Xデーに向けて場数を踏め。
+経験を積めば脳死で動けるようになる。</t>
+        </is>
+      </c>
+      <c r="C2215" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2215" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2215" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-08-24 (女を追うな)
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2215"/>
+  <dimension ref="A1:G2216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64389,6 +64389,35 @@
         </is>
       </c>
     </row>
+    <row r="2216">
+      <c r="A2216" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B2216" t="inlineStr">
+        <is>
+          <t>「女を追うな」という助言は一長一短。
+確かに、童貞チー牛や理想の女を抱けない層は、まずステータスを上げることに注力した方がいい。
+でも、ある程度レベルを上げたら、女を追わないと始まらない。
+ここを勘違いしてはいけない。
+「今の俺がモテるのは無理だな」と実感しているなら、全力で男磨きに取り組め。
+でも、ある程度自信がついたら現場に行け。
+実戦を繰り返せば、自分だけのノウハウを作れる。</t>
+        </is>
+      </c>
+      <c r="C2216" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2216" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2216" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-08-25: BMI post
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2216"/>
+  <dimension ref="A1:G2217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64418,6 +64418,29 @@
         </is>
       </c>
     </row>
+    <row r="2217">
+      <c r="A2217" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B2217" t="inlineStr">
+        <is>
+          <t>BMI＝筋トレ知らない奴がこだわる数字。</t>
+        </is>
+      </c>
+      <c r="C2217" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2217" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2217" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-08-25: 男磨き2種類
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2217"/>
+  <dimension ref="A1:G2218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64441,6 +64441,43 @@
         </is>
       </c>
     </row>
+    <row r="2218">
+      <c r="A2218" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B2218" t="inlineStr">
+        <is>
+          <t>男磨きには2種類ある。
+① 自己規律を作る男磨き
+↓
+やるべき人は自堕落、スマホ中毒、ゲーム中毒でモテる・モテない以前に「自分を律すること」ができていない男がやるもの。
+睡眠、運動習慣、瞑想、スマホ断ち、生活習慣の改善などの基礎習慣。
+まずはここで土台を作る。
+② 魅力度を上げる男磨き
+↓
+基礎習慣ができた上で、直接的に魅力を上げていく。
+肉体改造、金稼ぎ、髪、肌、服装、清潔感、姿勢、整形など。
+堕落している男は①が②をやる上で強力な土台になる。
+ニートでスマホ廃人の俺も①から始めた。
+自堕落な男は①から。
+土台ができた男は②へ。
+この2つを網羅して、あとは現場に出れば余裕で戦える。</t>
+        </is>
+      </c>
+      <c r="C2218" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2218" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2218" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-08-26: モテテク
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2219"/>
+  <dimension ref="A1:G2220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64512,6 +64512,36 @@
         </is>
       </c>
     </row>
+    <row r="2220">
+      <c r="A2220" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B2220" t="inlineStr">
+        <is>
+          <t>モテテクで個人的に効果的だったもの
+・ピークエンド
+・内面を褒める
+・フット・イン・ザ・ドア
+・名前を呼ぶ
+・ダブル・バインド
+(2つ選択肢を与える)
+「LINEの返信をわざと遅らせてマインドシェアを...」は、結果論だと思ってる。</t>
+        </is>
+      </c>
+      <c r="C2220" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2220" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2220" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-08-26: 単純接触効果
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2220"/>
+  <dimension ref="A1:G2221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64542,6 +64542,34 @@
         </is>
       </c>
     </row>
+    <row r="2221">
+      <c r="A2221" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B2221" t="inlineStr">
+        <is>
+          <t>モテテクにおける単純接触効果は、
+本体が魅力的であることが前提。
+チー牛が女に何回も接触したとて、
+マイナスイメージを増幅させるだけ。
+興味ゼロの広告がウザいのと同じ。
+女を追う前に己を磨け。</t>
+        </is>
+      </c>
+      <c r="C2221" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2221" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2221" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-08-26: 奢り奢られ論争
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2221"/>
+  <dimension ref="A1:G2222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64570,6 +64570,36 @@
         </is>
       </c>
     </row>
+    <row r="2222">
+      <c r="A2222" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B2222" t="inlineStr">
+        <is>
+          <t>奢り奢られ論争の、
+「奢りたくない女と飯屋に行かない」
+「男が稼いで、女は家事」
+みたいな意見には100%同意。
+あとは逆に相手が年上女性なら、あえて奢らせて「可愛がられポジション」に行くのもあり。
+割り勘が一番意味がない。
+奢るか、奢られるか。
+関係性に合わせて、どちらかに振り切れ。</t>
+        </is>
+      </c>
+      <c r="C2222" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2222" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2222" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add post 2026-08-27: 筋トレ中の飲み物
</commit_message>
<xml_diff>
--- a/x_posts/posts_categorized.xlsx
+++ b/x_posts/posts_categorized.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2222"/>
+  <dimension ref="A1:G2223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64600,6 +64600,34 @@
         </is>
       </c>
     </row>
+    <row r="2223">
+      <c r="A2223" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B2223" t="inlineStr">
+        <is>
+          <t>筋トレ中の飲み物は水で良い。
+理由はトレ前の食事を摂っていればエネルギー枯渇する事なんてないから。
+EAAを摂って損することはないけど、
+サプリの優先度的に低い。
+減量期に3時間トレする時なら話は別かもだけど。
+あとは強度確保のためにまともなプレ買った方がいい。</t>
+        </is>
+      </c>
+      <c r="C2223" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2223" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2223" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>